<commit_message>
Add Next.js app scaffold for Pertemuan6
Bootstrap a Next.js project under Pertemuan6. Added .gitignore, README, AGENTS.md, CLAUDE.md, ESLint and Next config files, package.json, postcss and tsconfig, public assets, and app sources (favicon, globals.css, layout.tsx, page.tsx). Also added an API route (src/app/api/berita/route.ts) and a simple DB helper (src/lib/db.ts). Updated the binary Pertemuan4/hasil_cleaning.xlsx. This provides an initial project scaffold, lint/build configuration, and a basic API/DB stub for further development.
</commit_message>
<xml_diff>
--- a/Pertemuan4/hasil_cleaning.xlsx
+++ b/Pertemuan4/hasil_cleaning.xlsx
@@ -455,301 +455,301 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Nah Loh! Selingkuhan Bill Gates Ternyata yang Kenalkan ke Epstein</t>
+          <t>Tak Sabar Tunggu GTA 6, Pria Ini Bikin Tiruannya Pakai AI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Nah Loh! Selingkuhan Bill Gates Ternyata yang Kenalkan ke Epstein</t>
+          <t>Tak Sabar Tunggu GTA 6, Pria Ini Bikin Tiruannya Pakai AI</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8525139/nah-loh-selingkuhan-bill-gates-ternyata-yang-kenalkan-ke-epstein</t>
+          <t>https://inet.detik.com/games-news/d-8534872/tak-sabar-tunggu-gta-6-pria-ini-bikin-tiruannya-pakai-ai</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8525139/nah-loh-selingkuhan-bill-gates-ternyata-yang-kenalkan-ke-epstein</t>
+          <t>https://inet.detik.com/games-news/d-8534872/tak-sabar-tunggu-gta-6-pria-ini-bikin-tiruannya-pakai-ai</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/02/05/bill-gates-1770250296944_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2025/05/07/rockstar-rilis-trailer-gta-6-yang-kedua-tampilkan-aksi-2-karakter-utama-1746583798227_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F2" s="1" t="n">
-        <v>46183.45809272666</v>
+        <v>46190.45775707352</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>14 Foto Foto Kelam Perang Dunia II, Bukti Nyata Kengerian yang Tak Terlupakan</t>
+          <t>15 Foto Hanya Mata Jeli yang Bisa Menemukan Sosok di Foto 'Penampakan' Ini</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>14 Foto Foto Kelam Perang Dunia II, Bukti Nyata Kengerian yang Tak Terlupakan</t>
+          <t>15 Foto Hanya Mata Jeli yang Bisa Menemukan Sosok di Foto 'Penampakan' Ini</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/fotoinet/d-8525552/foto-kelam-perang-dunia-ii-bukti-nyata-kengerian-yang-tak-terlupakan</t>
+          <t>https://inet.detik.com/fotoinet/d-8534856/hanya-mata-jeli-yang-bisa-menemukan-sosok-di-foto-penampakan-ini</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/fotoinet/d-8525552/foto-kelam-perang-dunia-ii-bukti-nyata-kengerian-yang-tak-terlupakan</t>
+          <t>https://inet.detik.com/fotoinet/d-8534856/hanya-mata-jeli-yang-bisa-menemukan-sosok-di-foto-penampakan-ini</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/10/foto-kelam-perang-1781055113755_43.webp?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/17/kumpulan-foto-unik-dengan-sosok-tersembunyi-yang-sulit-ditemukan-1781658346072_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F3" s="1" t="n">
-        <v>46183.45809272666</v>
+        <v>46190.45775707352</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>WhatsApp Cabut Dukungan untuk iOS Lawas Ini, Segera Update iPhone Kalian!</t>
+          <t>Haaland Menggila di Debut Piala Dunia 2026, Borong 2 Gol Bikin Heboh Medsos</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>WhatsApp Cabut Dukungan untuk iOS Lawas Ini, Segera Update iPhone Kalian!</t>
+          <t>Haaland Menggila di Debut Piala Dunia 2026, Borong 2 Gol Bikin Heboh Medsos</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/mobile-apps/d-8525537/whatsapp-cabut-dukungan-untuk-ios-lawas-ini-segera-update-iphone-kalian</t>
+          <t>https://inet.detik.com/cyberlife/d-8534834/haaland-menggila-di-debut-piala-dunia-2026-borong-2-gol-bikin-heboh-medsos</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/mobile-apps/d-8525537/whatsapp-cabut-dukungan-untuk-ios-lawas-ini-segera-update-iphone-kalian</t>
+          <t>https://inet.detik.com/cyberlife/d-8534834/haaland-menggila-di-debut-piala-dunia-2026-borong-2-gol-bikin-heboh-medsos</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/02/18/ilustrasi-whatsapp-1771389858556_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/17/irak-vs-norwegia-1781650428426_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F4" s="1" t="n">
-        <v>46183.45809272666</v>
+        <v>46190.45775707352</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Drama Siri AI di Eropa: Apple Salahkan DMA, UE Membalas</t>
+          <t>Gibran Ingatkan Bahaya AI, Singgung Teknologi Tanpa Etika Itu Berbahaya</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Drama Siri AI di Eropa: Apple Salahkan DMA, UE Membalas</t>
+          <t>Gibran Ingatkan Bahaya AI, Singgung Teknologi Tanpa Etika Itu Berbahaya</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/consumer/d-8525512/drama-siri-ai-di-eropa-apple-salahkan-dma-ue-membalas</t>
+          <t>https://inet.detik.com/law-and-policy/d-8534804/gibran-ingatkan-bahaya-ai-singgung-teknologi-tanpa-etika-itu-berbahaya</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/consumer/d-8525512/drama-siri-ai-di-eropa-apple-salahkan-dma-ue-membalas</t>
+          <t>https://inet.detik.com/law-and-policy/d-8534804/gibran-ingatkan-bahaya-ai-singgung-teknologi-tanpa-etika-itu-berbahaya</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/10/siri-ai-1781052453392_43.png?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/17/gibran-rakabuming-1781653746966_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F5" s="1" t="n">
-        <v>46183.45809272666</v>
+        <v>46190.45775707352</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Selingkuhan Bill Gates Curhat ke Epstein karena Melinda Tak Mau Akur</t>
+          <t>Mbappe Lampaui Messi di Piala Dunia, Netizen Doakan Pecahkan Rekor Klose</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Selingkuhan Bill Gates Curhat ke Epstein karena Melinda Tak Mau Akur</t>
+          <t>Mbappe Lampaui Messi di Piala Dunia, Netizen Doakan Pecahkan Rekor Klose</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8525496/selingkuhan-bill-gates-curhat-ke-epstein-karena-melinda-tak-mau-akur</t>
+          <t>https://inet.detik.com/cyberlife/d-8534801/mbappe-lampaui-messi-di-piala-dunia-netizen-doakan-pecahkan-rekor-klose</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8525496/selingkuhan-bill-gates-curhat-ke-epstein-karena-melinda-tak-mau-akur</t>
+          <t>https://inet.detik.com/cyberlife/d-8534801/mbappe-lampaui-messi-di-piala-dunia-netizen-doakan-pecahkan-rekor-klose</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2022/05/02/bill-gates-dan-melinda-gates_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/17/kylian-mbappe-1781642953407_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F6" s="1" t="n">
-        <v>46183.45809272666</v>
+        <v>46190.45775707352</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NASA Tancap Gas ke Bulan, Kru Artemis III Resmi Diperkenalkan</t>
+          <t>Ponsel Tak Lagi Jadi Raja? CEO Qualcomm Ungkap Penggantinya</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>NASA Tancap Gas ke Bulan, Kru Artemis III Resmi Diperkenalkan</t>
+          <t>Ponsel Tak Lagi Jadi Raja? CEO Qualcomm Ungkap Penggantinya</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/science/d-8525489/nasa-tancap-gas-ke-bulan-kru-artemis-iii-resmi-diperkenalkan</t>
+          <t>https://inet.detik.com/business/d-8534792/ponsel-tak-lagi-jadi-raja-ceo-qualcomm-ungkap-penggantinya</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/science/d-8525489/nasa-tancap-gas-ke-bulan-kru-artemis-iii-resmi-diperkenalkan</t>
+          <t>https://inet.detik.com/business/d-8534792/ponsel-tak-lagi-jadi-raja-ceo-qualcomm-ungkap-penggantinya</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/10/artemis-iii-1781049032759_43.webp?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2025/10/29/ilustrasi-kirim-chat-atau-pesan-via-whatsapp-wa-1761720050538_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F7" s="1" t="n">
-        <v>46183.45809272666</v>
+        <v>46190.45775707352</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Apple Rombak App Store di WWDC 2026, Pengembang Makin Cuan</t>
+          <t>Maskapai Israel Kerja Sama dengan Elon Musk, Pakai Starlink</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Apple Rombak App Store di WWDC 2026, Pengembang Makin Cuan</t>
+          <t>Maskapai Israel Kerja Sama dengan Elon Musk, Pakai Starlink</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8525478/apple-rombak-app-store-di-wwdc-2026-pengembang-makin-cuan</t>
+          <t>https://inet.detik.com/business/d-8534785/maskapai-israel-kerja-sama-dengan-elon-musk-pakai-starlink</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8525478/apple-rombak-app-store-di-wwdc-2026-pengembang-makin-cuan</t>
+          <t>https://inet.detik.com/business/d-8534785/maskapai-israel-kerja-sama-dengan-elon-musk-pakai-starlink</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/09/app-store-1780999382205_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2024/07/01/ilustrasi-pesawat-maskapai-israel-el-al-di-bandara-nice-prancis_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F8" s="1" t="n">
-        <v>46183.45809272666</v>
+        <v>46190.45775707352</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>6 Bintang Merah Mencurigakan Diduga Telan Banyak Planet</t>
+          <t>Video Pesan Wapres Gibran untuk Generasi Muda: Gunakan AI untuk Belajar</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>6 Bintang Merah Mencurigakan Diduga Telan Banyak Planet</t>
+          <t>Video Pesan Wapres Gibran untuk Generasi Muda: Gunakan AI untuk Belajar</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/science/d-8525153/6-bintang-merah-mencurigakan-diduga-telan-banyak-planet</t>
+          <t>https://inet.detik.com/detiktv/d-8534705/video-pesan-wapres-gibran-untuk-generasi-muda-gunakan-ai-untuk-belajar</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/science/d-8525153/6-bintang-merah-mencurigakan-diduga-telan-banyak-planet</t>
+          <t>https://inet.detik.com/detiktv/d-8534705/video-pesan-wapres-gibran-untuk-generasi-muda-gunakan-ai-untuk-belajar</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/09/bintang-merah-1780997486052_43.webp?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/16/wakil-presiden-gibran-rakabuming-raka-1781619885697_43.png?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F9" s="1" t="n">
-        <v>46183.45809272666</v>
+        <v>46190.45775707352</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Netflix, PUBG Hingga Shopee Sudah Lapor Penilaian Mandiri PP Tunas</t>
+          <t>Pesan Gibran ke Pelajar: Gunakan AI untuk Belajar, Bukan untuk Malas</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Netflix, PUBG Hingga Shopee Sudah Lapor Penilaian Mandiri PP Tunas</t>
+          <t>Pesan Gibran ke Pelajar: Gunakan AI untuk Belajar, Bukan untuk Malas</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/law-and-policy/d-8525332/netflix-pubg-hingga-shopee-sudah-lapor-penilaian-mandiri-pp-tunas</t>
+          <t>https://inet.detik.com/law-and-policy/d-8534667/pesan-gibran-ke-pelajar-gunakan-ai-untuk-belajar-bukan-untuk-malas</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/law-and-policy/d-8525332/netflix-pubg-hingga-shopee-sudah-lapor-penilaian-mandiri-pp-tunas</t>
+          <t>https://inet.detik.com/law-and-policy/d-8534667/pesan-gibran-ke-pelajar-gunakan-ai-untuk-belajar-bukan-untuk-malas</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/08/menkomdigi-meutya-hafid-1780905615359_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/16/wakil-presiden-gibran-rakabuming-raka-1781619885697_43.png?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F10" s="1" t="n">
-        <v>46183.45809272666</v>
+        <v>46190.45775707352</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Lintasarta Tetap Investasi AI di Tengah Pelemahan Rupiah dan Krisis Memori</t>
+          <t>Gibran: Indonesia Harus Jadi Penguasa AI, Bukan Sekedar Pengguna</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Lintasarta Tetap Investasi AI di Tengah Pelemahan Rupiah dan Krisis Memori</t>
+          <t>Gibran: Indonesia Harus Jadi Penguasa AI, Bukan Sekedar Pengguna</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/business/d-8525208/lintasarta-tetap-investasi-ai-di-tengah-pelemahan-rupiah-dan-krisis-memori</t>
+          <t>https://inet.detik.com/law-and-policy/d-8534648/gibran-indonesia-harus-jadi-penguasa-ai-bukan-sekedar-pengguna</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/business/d-8525208/lintasarta-tetap-investasi-ai-di-tengah-pelemahan-rupiah-dan-krisis-memori</t>
+          <t>https://inet.detik.com/law-and-policy/d-8534648/gibran-indonesia-harus-jadi-penguasa-ai-bukan-sekedar-pengguna</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/09/lintasarta-intelligent-core-1781009959965_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/16/wakil-presiden-gibran-rakabuming-raka-1781619885697_43.png?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F11" s="1" t="n">
-        <v>46183.45809272666</v>
+        <v>46190.45775707352</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: penambahan fitur anti duplikasi
</commit_message>
<xml_diff>
--- a/Pertemuan4/hasil_cleaning.xlsx
+++ b/Pertemuan4/hasil_cleaning.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,305 +451,360 @@
           <t>waktu_scraping</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>isi_berita</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tak Sabar Tunggu GTA 6, Pria Ini Bikin Tiruannya Pakai AI</t>
+          <t>10 Foto Lionel Messi Hattrick, Dipuji Setinggi Langit</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Tak Sabar Tunggu GTA 6, Pria Ini Bikin Tiruannya Pakai AI</t>
+          <t>10 Foto Lionel Messi Hattrick, Dipuji Setinggi Langit</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/games-news/d-8534872/tak-sabar-tunggu-gta-6-pria-ini-bikin-tiruannya-pakai-ai</t>
+          <t>https://inet.detik.com/fotoinet/d-8535031/lionel-messi-hattrick-dipuji-setinggi-langit</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/games-news/d-8534872/tak-sabar-tunggu-gta-6-pria-ini-bikin-tiruannya-pakai-ai</t>
+          <t>https://inet.detik.com/fotoinet/d-8535031/lionel-messi-hattrick-dipuji-setinggi-langit</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2025/05/07/rockstar-rilis-trailer-gta-6-yang-kedua-tampilkan-aksi-2-karakter-utama-1746583798227_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/17/meme-messi-1781666958944_43.png?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F2" s="1" t="n">
-        <v>46190.45775707352</v>
+        <v>46190.52412886219</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Jakarta - Lionel Messi mencetak hattrick dalam kemenangan Argentina atas Aljazair 3-0 di ajang Piala Dunia 2026. Dengan 3 gol yang disarangkan ke Aljazair, Lionel Messi menjadi pencetak gol terbanyak di Piala Dunia bersama Miroslav Klose. Foto: X.com Messi dan Klose di puncak dengan sama-sama melesakkan 17 gol sepanjang sejarah keikutsertaan mereka di Piala Dunia. Foto: X.com Memang benar-benar Lionel Messi adalah pesepakbola terbaik dunia sampai saat ini. Foto: X.com Sungguh penampilan klasik dari Messi. Foto: X.com Sudah berusia 38 tahun dan memenangkan segalanya, Messi tadi tetap ngotot bahkan membantu pertahanan. Foto: X.com Akun resmi Timnas Argentina memuji penampilan sang mega bintang. Foto: X.com Messi pun menjadi Man of The Match. Foto: X.com Berbagai rekor menakjubkan Messi di ajang Piala Dunia. Foto: X.com Sudah 20 tahun berlalu, Messi tetap luar biasa. Foto: X.com Para megabintang mulai bersinar di Piala Dunia 2026. Foto: X.com (/) TAGS lionel messi piala dunia 2026 LIHAT LAINNYA Tautan telah disalin</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>15 Foto Hanya Mata Jeli yang Bisa Menemukan Sosok di Foto 'Penampakan' Ini</t>
+          <t>Kampus Ini Sudah Lahirkan 12 Unicorn AI dan Hardware, Ada DJI di Baliknya</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>15 Foto Hanya Mata Jeli yang Bisa Menemukan Sosok di Foto 'Penampakan' Ini</t>
+          <t>Kampus Ini Sudah Lahirkan 12 Unicorn AI dan Hardware, Ada DJI di Baliknya</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/fotoinet/d-8534856/hanya-mata-jeli-yang-bisa-menemukan-sosok-di-foto-penampakan-ini</t>
+          <t>https://inet.detik.com/cyberlife/d-8534903/kampus-ini-sudah-lahirkan-12-unicorn-ai-dan-hardware-ada-dji-di-baliknya</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/fotoinet/d-8534856/hanya-mata-jeli-yang-bisa-menemukan-sosok-di-foto-penampakan-ini</t>
+          <t>https://inet.detik.com/cyberlife/d-8534903/kampus-ini-sudah-lahirkan-12-unicorn-ai-dan-hardware-ada-dji-di-baliknya</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/17/kumpulan-foto-unik-dengan-sosok-tersembunyi-yang-sulit-ditemukan-1781658346072_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/15/innox-1781527712161_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F3" s="1" t="n">
-        <v>46190.45775707352</v>
+        <v>46190.52412886219</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Jakarta - Jika Silicon Valley dikenal sebagai rumah bagi raksasa teknologi dunia, China memiliki Shenzhen sebagai pusat lahirnya inovasi hardware dan kecerdasan buatan (AI). Di kota inilah berdiri Shenzhen InnoX Academy, sebuah institusi yang dijuluki banyak kalangan sebagai "pabrik startup" karena berhasil melahirkan puluhan perusahaan teknologi dengan dampak global. Didirikan pada 2021 oleh Profesor Li Zexiang, akademisi dari Hong Kong University of Science and Technology (HKUST) yang juga dikenal sebagai salah satu tokoh di balik kesuksesan DJI, InnoX mengusung konsep berbeda dari kampus atau inkubator startup konvensional. Mereka menggabungkan pendidikan kewirausahaan, inkubasi startup, akselerasi manufaktur, hingga dukungan ekspansi global dalam satu ekosistem terintegrasi. "Rekam jejak Li Zexiang sendiri tidak main-main. Selama kariernya, ia telah membantu menginkubasi lebih dari 200 perusahaan smart hardware yang menghasilkan empat perusahaan publik dan 12 unicorn, termasuk DJI yang kini menjadi pemimpin pasar drone konsumen dunia," terang Carol Yu Founding Partner &amp; Senior Vice President InnoX. SCROLL TO CONTINUE WITH CONTENT ADVERTISEMENT Baca Juga : Baseus PicoGo Air Rilis, Powerbank Setipis Kartu Tantang Xiaomi UltraThin Sejak berdiri, InnoX telah menarik lebih dari 19.000 pendaftar dari berbagai negara dan mendukung hampir 1.000 entrepreneur melalui berbagai program inovasi dan inkubasi startup. Saat ini, sekitar 100 proyek startup sedang dibina, dengan lebih dari 80% berfokus pada pengembangan AI dan hardware untuk pasar global. Model yang diterapkan InnoX berfokus pada membantu inovator mengubah ide menjadi produk siap pasar. Para peserta tidak hanya belajar teori bisnis, tetapi juga menjalani proses lengkap mulai dari riset pengguna, perancangan produk, pengembangan teknologi, pembuatan prototipe, hingga strategi pemasaran global. Sosok Profesor Li Zexiang Foto: Innox Keunggulan terbesar InnoX terletak pada lokasinya yang berada di Shenzhen, kota yang dikenal sebagai pusat manufaktur teknologi dunia. Melalui jaringan lebih dari 1.600 pemasok dan mitra manufaktur, startup dapat mempercepat proses pengembangan produk, menguji berbagai prototipe, hingga melakukan produksi massal dengan lebih cepat dibanding banyak negara lain. Tak hanya membantu membangun produk, InnoX juga mendorong startup untuk langsung berpikir global sejak hari pertama. Lebih dari 80% startup binaannya memang dirancang untuk pasar internasional. Dukungan yang diberikan mencakup strategi crowdfunding, pameran teknologi internasional, branding, akses investor, hingga jaringan bisnis global. Carol Yu Founding Partner &amp; Senior Vice President InnoX. Foto: Innox Kekuatan ekosistem tersebut terlihat dari beragam startup yang lahir dari InnoX. Mulai dari Kamingo yang mampu mengubah sepeda biasa menjadi e-bike dalam hitungan detik, XBREW dengan mesin kopi nitro tanpa kartrid pertama di dunia, hingga Y-H2O yang mengembangkan kapal hydrofoil listrik futuristis. Ada pula Finnox yang mengembangkan AI untuk memahami emosi manusia, serta Lumi, robot lampu berbasis AI yang menghadirkan interaksi layaknya karakter animasi Pixar. Pada ajang BEYOND Expo 2026, InnoX membawa sekitar 30 startup AI dan hardware untuk memamerkan inovasi terbaru mereka di bidang robotika, mobilitas pintar, embodied AI, kesehatan digital, hingga perangkat gaya hidup cerdas. Untuk memperkuat ekosistem inovasinya, InnoX juga menjalin kolaborasi dengan lebih dari 20 universitas ternama dunia, termasuk Stanford University, Olin College of Engineering, King Abdullah University of Science and Technology (KAUST), University of Hong Kong, dan HKUST. Jaringan global tersebut membuka akses bagi para pendiri startup ke talenta, investor, industri, serta sumber daya manufaktur dari berbagai negara. Innox Foto: Innox Di tengah persaingan global membangun dominasi AI, Shenzhen InnoX Academy menunjukkan bahwa kesuksesan tidak hanya ditentukan oleh teknologi canggih, tetapi juga oleh ekosistem yang mampu mengubah ide menjadi produk yang benar-benar digunakan masyarakat. "Dari Shenzhen, berbagai startup AI dan hardware kini bersiap menembus pasar dunia," pungkas Yu. Baca Juga : Tamagotchi Kini Makin Pintar, Punya AI dan Bisa Pantau Tanaman Video AI Bikin Konsumsi Air Dunia Melejit: Dampaknya Bisa Kekeringan! Video AI Bikin Konsumsi Air Dunia Melejit: Dampaknya Bisa Kekeringan! (afr/afr) TAGS unicorn shenzhen innox academy dji innox academy kecerdasan buatan startup teknologi global connect show LIHAT LAINNYA Tautan telah disalin</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Haaland Menggila di Debut Piala Dunia 2026, Borong 2 Gol Bikin Heboh Medsos</t>
+          <t>Zuckerberg Bayar Rp 248 T untuk Bocah Ajaib, Hasilnya Belum Ada</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Haaland Menggila di Debut Piala Dunia 2026, Borong 2 Gol Bikin Heboh Medsos</t>
+          <t>Zuckerberg Bayar Rp 248 T untuk Bocah Ajaib, Hasilnya Belum Ada</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8534834/haaland-menggila-di-debut-piala-dunia-2026-borong-2-gol-bikin-heboh-medsos</t>
+          <t>https://inet.detik.com/business/d-8534912/zuckerberg-bayar-rp-248-t-untuk-bocah-ajaib-hasilnya-belum-ada</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8534834/haaland-menggila-di-debut-piala-dunia-2026-borong-2-gol-bikin-heboh-medsos</t>
+          <t>https://inet.detik.com/business/d-8534912/zuckerberg-bayar-rp-248-t-untuk-bocah-ajaib-hasilnya-belum-ada</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/17/irak-vs-norwegia-1781650428426_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2025/06/11/alexandr-wang-1749622991230_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F4" s="1" t="n">
-        <v>46190.45775707352</v>
+        <v>46190.52412886219</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Jakarta - Sekitar setahun lampau, MarkZuckerberg berinvestasi gila-gilaan untuk meningkatkan kemampuan kecerdasan buatan atau AI Meta, yang tertinggal jauh dari pesaing. Salah satunya dengan merekrut pakar AIAlexandr Wang yang menghabiskan USD 14 miliar (Rp 248 triliun). Uang itu diguyur untuk Scale AI, startup AI yang didirikan oleh Wang, anak muda yang baru berusia 29 tahun saat ini tapi dianggap sangat cerdas di bidang AI. Beberapa engineer Scale AI juga bergabung dengan Meta. Pencapaian besar Wang yang memimpin MetaSuperintelligence Labs adalah peluncuran model AI Muse Spark bulan April. Dengan produk itu, Meta setidaknya kembali diperhitungkan di ranah AI, meskipun masih tertinggal jauh di belakang OpenAI, Anthropic, dan Google. Namun demikian dari sisi finansial, hasilnya belum ada. SCROLL TO CONTINUE WITH CONTENT Kini CEO Mark Zuckerberg bertugas menjadikan kerja keras Wang sebagai kesuksesan finansial. Itu berarti menunjukkan perusahaan mampu menarik pengguna berbayar untuk AI-nya. Baca juga: Curhat Karyawan Meta yang Dipindah ke Divisi AI: Seperti Gulag "Meta perlu memberi lebih banyak bukti nyata terkait adopsi maupun komersialisasi. Investor menantikan Meta memonetisasi produk baru yang mengutamakan AI, di luar dampak positif substansial yang diberikan AI dalam menyempurnakan model periklanan," ujar Ralph Schackart, analis di William Blair yang dikutip detikINET dari CNBC. ADVERTISEMENT Wall Street juga sejauh ini tidak terkesan. Saham Meta anjlok 18% 12 bulan terakhir. Hal itu terjadi bahkan setelah Meta melaporkan pertumbuhan pendapatan 33% pada kuartal pertama. Meta awalnya terjun ke ranah AI dengan model Llama, menawarkan pendekatan open source yang memungkinkan pengembang mengutak-atik secara bebas, sementara pembuat AI lain memungut biaya. Ternyata model itu adalah blunder. April 2025, peluncuran Llama 4 gagal total, tak mampu memikat pengembang dan membuat Zuckerberg mempertimbangkan kembali pendekatan AI Meta. Dua bulan kemudian, Zuckerberg mengejutkan dunia teknologi dengan mengumumkan investasi USD 14,3 miliar untuk Scale AI dan mendatangkan Wang. Pengembangan dan peluncuran Muse Spark oleh Wang pada bulan April tahun ini mulai menggerakkan roda perusahaan. Model baru ini dirancang mudah diintegrasikan ke aplikasi Meta seperti Facebook dan Instagram, serta perangkat AI seperti kacamata Ray-Ban Meta. Sebaik apapun model Wang, jalan Zuckerberg terjal setelah kegagalan Llama. "Saya rasa komunitas AI sebagian besar mengabaikan Meta pada titik ini," ujar Rob May, CEO startup Neurometric. Andrew Moore, CEO startup korporat Lovelace dan mantan kepala AI Google Cloud, mengatakan belum terlambat bagi Meta untuk menemukan jalurnya. Meta harus menunjukkan keunggulan di suatu area AI, entah itu pada biaya atau nuansa teknis lainnya yang penting bagi para pengembang. Masalah lain adalah kemerosotan moral kerja. Meta baru saja memecat sekitar 8.000 pekerja. Terdapat pula ketegangan di petinggi organisasi AI tersebut. Meskipun perilisan Muse Spark dinilai tinggi secara internal, ada tekanan yang dialami Wang bersama mantan CEO GitHub Nat Friedman, yang juga bergabung dengan Meta. Namun dalam podcast bulan Mei, Wang menepis konflik internal. Wang menyebut Muse Spark sebagai 'makanan pembuka"'untuk apa yang akan datang, dan mengatakan bahwa akan ada model-model yang lebih kuat. Baca juga: Pentolan AI Amerika Ramai Pindah ke China, Ada Apa? Video Top 5: TAEMIN Masuk Grammy Museum-Zuckerberg Jadi Penasihat Trump Video Top 5: TAEMIN Masuk Grammy Museum-Zuckerberg Jadi Penasihat Trump (fyk/fyk) TAGS mark zuckerberg alexandr wang LIHAT LAINNYA Tautan telah disalin</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Gibran Ingatkan Bahaya AI, Singgung Teknologi Tanpa Etika Itu Berbahaya</t>
+          <t>WhatsApp di iPhone Kini Bisa Pakai 2 Nomor Sekaligus, Begini Caranya</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Gibran Ingatkan Bahaya AI, Singgung Teknologi Tanpa Etika Itu Berbahaya</t>
+          <t>WhatsApp di iPhone Kini Bisa Pakai 2 Nomor Sekaligus, Begini Caranya</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/law-and-policy/d-8534804/gibran-ingatkan-bahaya-ai-singgung-teknologi-tanpa-etika-itu-berbahaya</t>
+          <t>https://inet.detik.com/consumer/d-8534891/whatsapp-di-iphone-kini-bisa-pakai-2-nomor-sekaligus-begini-caranya</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/law-and-policy/d-8534804/gibran-ingatkan-bahaya-ai-singgung-teknologi-tanpa-etika-itu-berbahaya</t>
+          <t>https://inet.detik.com/consumer/d-8534891/whatsapp-di-iphone-kini-bisa-pakai-2-nomor-sekaligus-begini-caranya</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/17/gibran-rakabuming-1781653746966_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2025/05/30/ilustrasi-menggunakan-smartphone-atau-whataapp-1748579035406_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F5" s="1" t="n">
-        <v>46190.45775707352</v>
+        <v>46190.52412886219</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Daftar Isi Cara Menambahkan Akun WhatsApp Kedua di iPhone Cara Beralih Antar Akun Keunggulan Fitur Multi-Akun WhatsApp Jakarta - abar gembira bagi pengguna iPhone. WhatsApp kini resmi menghadirkan fitur multi-akun di iOS yang memungkinkan pengguna menggunakan dua nomor telepon berbeda dalam satu aplikasi WhatsApp. Sebelumnya, pengguna iPhone yang ingin memakai dua akun WhatsApp biasanya harus mengandalkan WhatsApp Business atau aplikasi pihak ketiga. Kini, WhatsApp menghadirkan solusi resmi yang lebih praktis, aman, dan mudah digunakan. Fitur ini sangat berguna bagi pengguna yang ingin memisahkan akun pribadi dan pekerjaan tanpa harus berganti perangkat atau memasang aplikasi tambahan. Seluruh chat, notifikasi, hingga pengaturan privasi masing-masing akun akan tetap terpisah. SCROLL TO CONTINUE WITH CONTENT ADVERTISEMENT Baca Juga : WhatsApp Cabut Dukungan untuk iOS Lawas Ini, Segera Update iPhone Kalian! Dengan hadirnya fitur multi-akun, pengguna cukup berpindah akun langsung dari aplikasi WhatsApp tanpa perlu login dan logout berulang kali. Sebelum mencoba fitur ini, ada beberapa syarat yang perlu dipenuhi. Pengguna harus menggunakan WhatsApp versi terbaru yang sudah mendukung multi-akun di iOS. Selain itu, diperlukan dua nomor telepon aktif yang bisa berasal dari kombinasi SIM fisik dan eSIM, atau dua eSIM sekaligus. Cara Menambahkan Akun WhatsApp Kedua di iPhone Bagi yang ingin mencoba, berikut langkah-langkah menambahkan akun WhatsApp kedua di iPhone: Buka aplikasi WhatsApp di iPhone. Masuk ke menu Pengaturan (Settings). Ketuk bagian profil yang menampilkan nama dan nomor telepon. Pilih opsi Tambahkan Akun (Add Account). Masukkan nomor telepon kedua yang ingin digunakan. Lakukan proses verifikasi melalui SMS atau panggilan suara. Masukkan kode verifikasi yang diterima. Setelah proses selesai, akun kedua akan langsung aktif di aplikasi WhatsApp. Pengguna kini dapat menggunakan dua akun WhatsApp berbeda dalam satu aplikasi tanpa perlu menginstal aplikasi tambahan. Cara Beralih Antar Akun WhatsApp juga membuat proses perpindahan akun menjadi sangat mudah. Untuk berpindah akun: Buka menu Settings. Pada bagian atas akan muncul daftar akun yang aktif. Pilih akun yang ingin digunakan. Selain itu, pengguna juga bisa menekan lama tab Settings untuk berpindah akun dengan lebih cepat. Setiap akun memiliki pengaturan sendiri, termasuk notifikasi, status, foto profil, pengaturan privasi, hingga cadangan chat. Dengan begitu, aktivitas pribadi dan pekerjaan tetap dapat dipisahkan dengan rapi. Keunggulan Fitur Multi-Akun WhatsApp Kehadiran fitur ini membawa sejumlah keuntungan bagi pengguna iPhone, di antaranya: Tidak perlu lagi menggunakan aplikasi pihak ketiga yang berisiko terhadap keamanan data. Notifikasi untuk masing-masing akun tetap terpisah. Pengaturan privasi dapat diatur berbeda untuk setiap akun. Status, foto profil, dan tema bisa dikelola secara independen. Didukung langsung oleh WhatsApp sehingga lebih aman dan stabil. Meski demikian, ada beberapa hal yang perlu diperhatikan. Setiap akun tetap membutuhkan nomor telepon yang berbeda karena satu nomor hanya dapat digunakan untuk satu akun WhatsApp. Selain itu, fitur multi-akun diluncurkan secara bertahap. Jika opsi Tambahkan Akun belum muncul di perangkat, pengguna disarankan memperbarui aplikasi WhatsApp melalui App Store dan menunggu distribusi fitur tersedia untuk seluruh pengguna. Dengan hadirnya fitur multi-akun resmi di iPhone, pengguna kini dapat mengelola dua nomor WhatsApp dalam satu aplikasi secara lebih praktis. Fitur ini menjadi solusi yang selama ini ditunggu banyak pengguna iPhone yang ingin memisahkan urusan pribadi dan pekerjaan tanpa ribet. Baca Juga : WhatsApp Garap Fitur Scam Alert untuk Hindarkan Pengguna dari Penipuan Video: Instagram, Facebook, sampai WhatsApp Nggak Full Gratis Lagi? Video: Instagram, Facebook, sampai WhatsApp Nggak Full Gratis Lagi? (afr/afr) TAGS whatsapp iphone aplikasi whatsapp fitur baru whatsapp multi akun whatsapp LIHAT LAINNYA Tautan telah disalin</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Mbappe Lampaui Messi di Piala Dunia, Netizen Doakan Pecahkan Rekor Klose</t>
+          <t>Tak Sabar Tunggu GTA 6, Pria Ini Bikin Tiruannya Pakai AI</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Mbappe Lampaui Messi di Piala Dunia, Netizen Doakan Pecahkan Rekor Klose</t>
+          <t>Tak Sabar Tunggu GTA 6, Pria Ini Bikin Tiruannya Pakai AI</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8534801/mbappe-lampaui-messi-di-piala-dunia-netizen-doakan-pecahkan-rekor-klose</t>
+          <t>https://inet.detik.com/games-news/d-8534872/tak-sabar-tunggu-gta-6-pria-ini-bikin-tiruannya-pakai-ai</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8534801/mbappe-lampaui-messi-di-piala-dunia-netizen-doakan-pecahkan-rekor-klose</t>
+          <t>https://inet.detik.com/games-news/d-8534872/tak-sabar-tunggu-gta-6-pria-ini-bikin-tiruannya-pakai-ai</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/17/kylian-mbappe-1781642953407_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2025/05/07/rockstar-rilis-trailer-gta-6-yang-kedua-tampilkan-aksi-2-karakter-utama-1746583798227_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F6" s="1" t="n">
-        <v>46190.45775707352</v>
+        <v>46190.52412886219</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Jakarta - Grand Theft Auto (GTA) 6 dijadwalkan meluncur pada November 2026 setelah dikembangkan kurang lebih satu dekade. Namun, seorang pendiri startup sudah tidak sabar menunggu lebih lama dan memutuskan membuat game tiruan GTA 6 dengan bantuan AI. Ziwen Xu, pendiri startup Hyperecho, belum lama ini mengumumkan rencananya untuk membuat GTA 6 versinya sendiri dengan teknik vibe coding. Ia menggunakan Claude 20x, model AI generatif paling canggih dari Anthropic yang tersedia untuk publik. Proyek itu dimulainya pada 11 Juni kemarin. Sejak saat itu, Xu terus membagikan update terbaru tentang kemajuan proyeknya dan membagikan kodenya di GitHub jika ada orang lain yang ingin melanjutkan proyeknya. SCROLL TO CONTINUE WITH CONTENT Baca Juga : Demi Info Terbaru Game GTA 6, YouTuber Mau Bobol Kantor Rockstar "Targetnya: mengalahkan peluncuran GTA 6 yang sebenarnya. Ambisius, mungkin bodoh, tapi saya tetap akan melakukannya," tulis Xu dalam postingannya di X, seperti dikutip dari Gizmodo, Rabu (17/6/2026). ADVERTISEMENT [Gambas:Twitter] Postingan yang diunggah Xu di X menyertakan cuplikan video singkat dari game tersebut. Pada hari pertama, sebagian besar cuplikan gameplay-nya hanya terdiri dari oval biru 3D yang bergerak dan melompat-lompat di dekat balok abu-abu. Di hari kedua, Xu mengunggah video baru yang menunjukkan karakter yang bentuknya mulai mirip seperti manusia sedang berlarian di lanskap perkotaan. Namun, Xu mengakui bahwa itu masih jauh dari sempurna. "Agen AI membangun gedung pencakar langit di pusat kota LA, yang jadi masalah besar, karena (game) ini seharusnya di Florida," tulis Xu. "Selain itu, saya telah menghabiskan 33% dari penggunaan mingguan 20x saya dalam satu hari. Jadi waktu terus berjalan," sambungnya. Hari keenam setelah proyek ini dimulai, game buatan Xu sudah terlihat lebih ekspansif dengan karakter NPC yang berjalan-jalan, mobil di jalanan, dan bahkan senjata. GTA 6 baru akan diluncurkan pada bulan November, jadi Xu masih memiliki beberapa bulan untuk menyelesaikan proyek game-nya dan mengalahkan developer Rockstar Games. Belum diketahui sejauh mana komitmen Xu untuk melanjutkan proyek game ini. Baca Juga : GTA 6 Dominasi November 2026, Banyak Game Besar Pilih Menjauh Video Pesan Wapres Gibran untuk Generasi Muda: Gunakan AI untuk Belajar Video Pesan Wapres Gibran untuk Generasi Muda: Gunakan AI untuk Belajar (vmp/afr) TAGS gta 6 ai vibe coding LIHAT LAINNYA Tautan telah disalin</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ponsel Tak Lagi Jadi Raja? CEO Qualcomm Ungkap Penggantinya</t>
+          <t>15 Foto Hanya Mata Jeli yang Bisa Menemukan Sosok di Foto 'Penampakan' Ini</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ponsel Tak Lagi Jadi Raja? CEO Qualcomm Ungkap Penggantinya</t>
+          <t>15 Foto Hanya Mata Jeli yang Bisa Menemukan Sosok di Foto 'Penampakan' Ini</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/business/d-8534792/ponsel-tak-lagi-jadi-raja-ceo-qualcomm-ungkap-penggantinya</t>
+          <t>https://inet.detik.com/fotoinet/d-8534856/hanya-mata-jeli-yang-bisa-menemukan-sosok-di-foto-penampakan-ini</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/business/d-8534792/ponsel-tak-lagi-jadi-raja-ceo-qualcomm-ungkap-penggantinya</t>
+          <t>https://inet.detik.com/fotoinet/d-8534856/hanya-mata-jeli-yang-bisa-menemukan-sosok-di-foto-penampakan-ini</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2025/10/29/ilustrasi-kirim-chat-atau-pesan-via-whatsapp-wa-1761720050538_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/17/kumpulan-foto-unik-dengan-sosok-tersembunyi-yang-sulit-ditemukan-1781658346072_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F7" s="1" t="n">
-        <v>46190.45775707352</v>
+        <v>46190.52412886219</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Jakarta - Kumpulan foto unik dengan sosok tersembunyi yang sulit ditemukan. Uji ketelitian mata dan lihat apakah kamu bisa menemukannya lebih cepat dari orang lain. Pemilik rumah ini mengaku akhirnya berhasil membeli rumah impiannya setelah bertahun-tahun menabung. Namun ada satu detail aneh di dapur mungil ini yang langsung menarik perhatian netizen. Apakah kamu menemukannya? Foto: Boredpanda Sekilas hanya terlihat kebun biasa yang dipenuhi rumput liar. Padahal ada seekor hewan yang bersembunyi dengan kamuflase nyaris sempurna di dalam foto ini. Foto: Boredpanda Foto ruang kuliah ini tampak normal, tetapi ada satu sosok yang membuat banyak orang harus melihatnya dua kali sebelum sadar apa yang sebenarnya terjadi. Foto: Boredpanda Batuan bersalju ini terlihat seperti tebing biasa. Namun jika diamati lebih teliti, ada penghuni liar yang menyatu hampir sempurna dengan lingkungan sekitarnya. Foto: Boredpanda Tas ransel hitam ini sukses membuat banyak orang bingung. Bukan karena bentuknya, melainkan karena ada sesuatu yang tersembunyi di dekatnya. Foto: Boredpanda Ekskavator CAT ini tampak seperti alat berat biasa yang sedang diparkir. Namun ada hewan berhasil bersembunyi di tempat yang tidak terduga. Foto: Boredpanda Rimbunnya daun bambu membuat objek tersembunyi dan berbahaya dalam foto ini sangat sulit ditemukan. Hanya mata yang benar-benar jeli yang bisa melihatnya dalam hitungan detik. Foto: Boredpanda Tumpukan kaus kaki ini ternyata menyimpan kejutan. Ada sepasang mata yang mengintip dari balik lipatan kain dan membuat foto ini viral. Foto: Boredpanda Pemandangan desa yang indah dari udara ini menyimpan satu objek yang tidak seharusnya ada di sana. Banyak orang baru menyadarinya setelah diperbesar. Foto: Boredpanda Hutan kering ini tampak kosong tanpa penghuni. Faktanya, ada seekor hewan yang sedang mengawasi kamera sambil berkamuflase dengan sangat baik. Foto: Boredpanda Kucing hitam ini sebenarnya tidak sendirian. Banyak orang baru menyadarinya setelah melihat bagian matanya yang menyala. Foto: Boredpanda Pagar kayu dan tanaman rambat tampak biasa saja. Tapi ada seekor ular yang berkamuflase begitu sempurna hingga sulit ditemukan dalam sekali pandang. Foto: Boredpanda Daun hijau ini menyimpan penghuni tersembunyi yang nyaris tak terlihat. Bentuk dan warnanya begitu mirip dengan daun tempat ia hinggap. Foto: Boredpanda Seorang pedagang roti sedang melayani pelanggan di pinggir jalan. Namun ada 'penjaga toko' tak terduga yang bersembunyi di etalase dan membuat banyak orang tertipu. Foto: Boredpanda Hamparan bebatuan dan dedaunan kering ini ternyata bukan sekadar pemandangan hutan biasa. Seekor ular besar bersembunyi di depan kamera dengan kamuflase yang luar biasa. Foto: Boredpanda (/) TAGS fotoinet fotodetikcom LIHAT LAINNYA Tautan telah disalin</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Maskapai Israel Kerja Sama dengan Elon Musk, Pakai Starlink</t>
+          <t>Haaland Menggila di Debut Piala Dunia 2026, Borong 2 Gol Bikin Heboh Medsos</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Maskapai Israel Kerja Sama dengan Elon Musk, Pakai Starlink</t>
+          <t>Haaland Menggila di Debut Piala Dunia 2026, Borong 2 Gol Bikin Heboh Medsos</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/business/d-8534785/maskapai-israel-kerja-sama-dengan-elon-musk-pakai-starlink</t>
+          <t>https://inet.detik.com/cyberlife/d-8534834/haaland-menggila-di-debut-piala-dunia-2026-borong-2-gol-bikin-heboh-medsos</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/business/d-8534785/maskapai-israel-kerja-sama-dengan-elon-musk-pakai-starlink</t>
+          <t>https://inet.detik.com/cyberlife/d-8534834/haaland-menggila-di-debut-piala-dunia-2026-borong-2-gol-bikin-heboh-medsos</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2024/07/01/ilustrasi-pesawat-maskapai-israel-el-al-di-bandara-nice-prancis_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/17/irak-vs-norwegia-1781650428426_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F8" s="1" t="n">
-        <v>46190.45775707352</v>
+        <v>46190.52412886219</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Jakarta - Erling Haaland akhirnya mencatatkan debut yang sangat dinanti di Piala Dunia 2026. Striker andalan Norwegia itu langsung tampil menggila dengan mencetak dua gol saat membantu timnya meraih kemenangan meyakinkan 4-1 atas Irak pada laga Grup I. Penampilan Haaland langsung menjadi sorotan dunia sepak bola. Bomber Manchester City tersebut menunjukkan mengapa dirinya dianggap sebagai salah satu penyerang paling berbahaya di generasi saat ini. Dua gol yang dicetaknya membuat pertahanan lawan tak berkutik dan membawa Norwegia membuka langkah di Piala Dunia dengan hasil sempurna. Tak pelak media sosial ikut heboh membahas aksi sang striker yang untuk pertama kalinya tampil di ajang sepak bola paling bergengsi di dunia. SCROLL TO CONTINUE WITH CONTENT ADVERTISEMENT Baca Juga : Mbappe Lampaui Messi di Piala Dunia, Netizen Doakan Pecahkan Rekor Klose Tak butuh waktu lama, nama Haaland langsung merajai trending topic di berbagai platform media sosial. Warganet dari berbagai negara ramai membahas aksi sang striker yang langsung mencetak brace pada penampilan pertamanya di Piala Dunia. [Gambas:Twitter] Di X, ribuan komentar memuji ketajaman pemain berusia 25 tahun tersebut. "Mungkin Haaland bisa aja jadi top score nih," kata @Muhammad_MARG. "Monster memang. Kalo butuh striker yang ahli finishing, tipe kaya haland ini yang paling bagus. Fisik oke, finishing juga oke. Jadi kombinasi yang bisa nyusahin lawan. Striker yang pas flop pun minimal cetak 25+ gol semusim," ujar @primas110. "Keren banget emang terminator satu ini," puji @kawulabolaid. "Debut Piala Dunia? Dua gol dan tiga poin. Haaland tak membuang waktu untuk memperkenalkan dirinya kepada dunia. Panggung Piala Dunia adalah satu-satunya yang kurang dalam catatan prestasinya. Ia sudah mulai menebus waktu yang hilang," tulis @abi_mat1 Video cuplikan dua gol Haaland juga viral di TikTok dan Instagram. Berbagai editan video dengan musik dramatis serta julukan "The Cyborg" membanjiri lini masa dan mengumpulkan jutaan tayangan hanya dalam hitungan jam. Kemenangan atas Irak menjadi modal berharga bagi Norwegia untuk melangkah ke fase berikutnya. Kehadiran Haaland membuat harapan publik Norwegia semakin tinggi setelah sekian lama tim nasional mereka jarang menjadi sorotan di panggung dunia. Jika mampu mempertahankan performa seperti ini, bukan tidak mungkin Haaland akan menjadi salah satu bintang terbesar turnamen sekaligus pesaing serius dalam perebutan gelar top skor. Baca Juga : Arab Saudi Tahan Uruguay, Netizen: Tutorial Kalahkan Arab Ada di Timnas Indonesia Video: Norwegia Lolos ke Piala Dunia 2026, Kalahkan Italia 4-1 Video: Norwegia Lolos ke Piala Dunia 2026, Kalahkan Italia 4-1 (afr/afr) TAGS haaland piala dunia 2026 gol haaland norwegia trending topic media sosial manchester city LIHAT LAINNYA Tautan telah disalin</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Video Pesan Wapres Gibran untuk Generasi Muda: Gunakan AI untuk Belajar</t>
+          <t>Gibran Ingatkan Bahaya AI, Singgung Teknologi Tanpa Etika Itu Berbahaya</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Video Pesan Wapres Gibran untuk Generasi Muda: Gunakan AI untuk Belajar</t>
+          <t>Gibran Ingatkan Bahaya AI, Singgung Teknologi Tanpa Etika Itu Berbahaya</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/detiktv/d-8534705/video-pesan-wapres-gibran-untuk-generasi-muda-gunakan-ai-untuk-belajar</t>
+          <t>https://inet.detik.com/law-and-policy/d-8534804/gibran-ingatkan-bahaya-ai-singgung-teknologi-tanpa-etika-itu-berbahaya</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/detiktv/d-8534705/video-pesan-wapres-gibran-untuk-generasi-muda-gunakan-ai-untuk-belajar</t>
+          <t>https://inet.detik.com/law-and-policy/d-8534804/gibran-ingatkan-bahaya-ai-singgung-teknologi-tanpa-etika-itu-berbahaya</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/16/wakil-presiden-gibran-rakabuming-raka-1781619885697_43.png?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/17/gibran-rakabuming-1781653746966_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F9" s="1" t="n">
-        <v>46190.45775707352</v>
+        <v>46190.52412886219</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Jakarta - Wakil Presiden Gibran Rakabuming Raka mengingatkan bahwa pesatnya perkembangan kecerdasan buatan atau Artificial Intelligence (AI) harus diiringi dengan penerapan etika yang kuat. Di tengah semakin luasnya pemanfaatan AI di berbagai bidang, Gibran menilai masyarakat perlu memahami bahwa teknologi bukan hanya soal kemampuan teknis, tetapi juga soal nilai dan integritas dalam penggunaannya. Meski menekankan Indonesia harus menguasai teknologi AI di masa mendatang, namun ia menyoroti ada hal utama yang dikedepankan terkait teknologi canggih ini, yakni terkait etika. SCROLL TO CONTINUE WITH CONTENT ADVERTISEMENT Baca Juga : Pesan Gibran ke Pelajar: Gunakan AI untuk Belajar, Bukan untuk Malas "Ada satu hal yang jauh lebih penting dari sekedar teknis penguasaan AI, yaitu etika. Teknologi tanpa etika itu berbahaya," kata Gibran seperti dikutip dari akun Instagram miliknya gibran_rakabuming, Rabu (17/6/2026). Ia menjelaskan AI memiliki potensi besar untuk membantu manusia menciptakan berbagai inovasi dan konten positif. Namun di sisi lain, teknologi yang sama juga dapat disalahgunakan untuk menyebarkan informasi palsu, melakukan plagiarisme, hingga melanggar privasi orang lain. "AI bisa digunakan untuk membuat konten positif, tapi juga bisa dipakai untuk menyebar hoax, melakukan plagiarisme, atau melanggar privasi orang lain," ucapnya. Gibran mengingatkan generasi muda agar tidak menggunakan AI untuk tindakan yang merugikan orang lain, melainkan kecanggihan teknologi harus dimanfaatkan untuk memberikan manfaat bagi masyarakat, bukan sebaliknya. "Saya ingin mengingatkan, pemanfaatan AI harus didasari oleh nilai-nilai integritas. Jangan gunakan AI untuk menipu. Jangan gunakan AI untuk menjatuhkan orang lain," tegasnya. Gibran Rakabuming, Wakil Presiden RI Foto: YouTube/@GibranTV Gibran menilai tantangan terbesar dalam era AI bukan hanya bagaimana masyarakat menguasai teknologi tersebut, tetapi juga bagaimana memastikan teknologi digunakan secara bertanggung jawab. "AI harus digunakan untuk kesejahteraan bersama, untuk mempermudah hidup, bukan untuk menciptakan kekacauan sosial. Kemajuan teknologi harus berjalan beriringan dengan kemajuan moralitas kita sebagai bangsa yang beradab," katanya. Dalam kesempatan tersebut, Gibran menyebut Indonesia memiliki talenta-talenta terbaik di bidang AI. Untuk itu, dikatanya, pemerintah menyiapkan ekosistemnya. Gibran juga menyinggung langkah pemerintah dalam menyiapkan tata kelola AI yang bertanggung jawab, yakni Indonesia telah menyelesaikan Readiness Assessment Methodology (RAM) AI yang disusun UNESCO sebagai instrumen untuk menilai kesiapan sekaligus tata kelola AI nasional. "Kuasai teknologinya. Pegang teguh etikanya. Mari kita jadikan AI sebagai jembatan menuju Indonesia yang lebih maju, lebih cerdas, dan lebih bermartabat," pungkasnya. Baca Juga : Gibran: Indonesia Harus Jadi Penguasa AI, Bukan Sekedar Pengguna Video Pesan Wapres Gibran untuk Generasi Muda: Gunakan AI untuk Belajar Video Pesan Wapres Gibran untuk Generasi Muda: Gunakan AI untuk Belajar (agt/afr) TAGS gibran rakabuming gibran rakabuming raka etika ai kecerdasan buatan ai etika teknologi LIHAT LAINNYA Tautan telah disalin</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Pesan Gibran ke Pelajar: Gunakan AI untuk Belajar, Bukan untuk Malas</t>
+          <t>Mbappe Lampaui Messi di Piala Dunia, Netizen Doakan Pecahkan Rekor Klose</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Pesan Gibran ke Pelajar: Gunakan AI untuk Belajar, Bukan untuk Malas</t>
+          <t>Mbappe Lampaui Messi di Piala Dunia, Netizen Doakan Pecahkan Rekor Klose</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/law-and-policy/d-8534667/pesan-gibran-ke-pelajar-gunakan-ai-untuk-belajar-bukan-untuk-malas</t>
+          <t>https://inet.detik.com/cyberlife/d-8534801/mbappe-lampaui-messi-di-piala-dunia-netizen-doakan-pecahkan-rekor-klose</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/law-and-policy/d-8534667/pesan-gibran-ke-pelajar-gunakan-ai-untuk-belajar-bukan-untuk-malas</t>
+          <t>https://inet.detik.com/cyberlife/d-8534801/mbappe-lampaui-messi-di-piala-dunia-netizen-doakan-pecahkan-rekor-klose</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/16/wakil-presiden-gibran-rakabuming-raka-1781619885697_43.png?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/17/kylian-mbappe-1781642953407_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F10" s="1" t="n">
-        <v>46190.45775707352</v>
+        <v>46190.52412886219</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Jakarta - Kylian Mbappe kembali membuktikan dirinya sebagai salah satu pemain terbaik dunia saat ini. Penyerang Timnas Prancis itu mencetak dua gol dalam kemenangan 3-1 atas Senegal pada laga pembuka Grup I Piala Dunia 2026, Rabu (17/6/2026) dini hari WIB. Brace tersebut bukan sekadar membantu Les Bleus meraih tiga poin penting. Mbappe juga resmi mencatatkan namanya dalam sejarah sebagai pencetak gol terbanyak Timnas Prancis di ajang Piala Dunia. Dua gol ke gawang Senegal membuat koleksi gol Mbappe di Piala Dunia mencapai 14 gol. Catatan itu membuatnya melampaui sejumlah legenda sepak bola dunia, termasuk Lionel Messi, sekaligus menyamai torehan legenda Jerman, Gerd M ller. SCROLL TO CONTINUE WITH CONTENT Baca Juga : Arab Saudi Tahan Uruguay, Netizen: Tutorial Kalahkan Arab Ada di Timnas Indonesia ADVERTISEMENT Kini, pemain berusia 27 tahun itu hanya terpaut dua gol dari Ronaldo Naz rio yang mengoleksi 15 gol dan tiga gol dari pemegang rekor sepanjang masa Piala Dunia, Miroslav Klose, dengan 16 gol. Tak hanya itu, dua gol ke gawang Senegal juga mengantarkan Mbappe mengoleksi 58 gol untuk Timnas Prancis. Jumlah tersebut membuatnya melampaui rekor Olivier Giroud sebagai pencetak gol terbanyak sepanjang sejarah Les Bleus. Gol ke gawang Senegal juga membuat Mbappe memperpanjang rekor uniknya. Ia kini berhasil mencetak gol dalam tiga edisi Piala Dunia secara beruntun, yakni 2018, 2022, dan 2026. Dengan format baru Piala Dunia yang diikuti 48 negara, setiap tim berpeluang memainkan lebih banyak pertandingan dibanding edisi sebelumnya. Situasi ini menjadi keuntungan tersendiri bagi Mbapp dalam perburuan rekor gol sepanjang masa. [Gambas:Twitter] Medsos Dibanjiri Pujian Penampilan gemilang sang kapten langsung memicu reaksi besar di media sosial. Nama Mbapp menjadi salah satu topik yang ramai diperbincangkan usai laga hingga masuk daftar trending topic dunia. Banyak penggemar menyebutnya sebagai pemain yang sedang menuju status legenda sepak bola dunia. Banyak yang mendoakan Mbappe memecahkan rekor terbanyak di dunia sepanjang masa. "3 GOL lagi melampaui gol Misroslav Klose dan jadi pencetak gol terbanyak Pildun sepanjang masa!," ujar @naufaldzimam. "Messi sama ronaldo bener2 ga ada apa2nya dibanding mbappe kalo urusan performa di piala dunia. Messi paling top di 2014. Mbappe ni kayaknya bakal 3x turnamen 3x menggila," kata @nararay__. "Gile baru 27 tahun udah jadi topskor Prancis sepanjang masa, kalo melangkah jauh di pildun ini bisa lewatin gol nya klose juga nih," ucap @hendrasumar. "Gap Klose-Mbapp tinggal 2 gol aja , perancis punya mesin gol yg nggak main main ," kata @Suri_Ethan. Kylian Mbapp mencetak dua gol saat Prancis mengalahkan Senegal 3-1 Foto: Getty Images/Dan Mullan Jika Prancis mampu melaju hingga babak akhir turnamen, Mbapp berpotensi menambah koleksi golnya dan melampaui catatan Miroslav Klose yang selama ini dianggap sulit disentuh. Melihat usianya yang masih 27 tahun, peluang Mbapp bahkan tidak hanya terbuka di Piala Dunia 2026. Ia masih berpotensi tampil pada edisi berikutnya dan memperlebar rekor tersebut. Setelah menjadi juara dunia pada 2018, meraih Sepatu Emas pada 2022, dan kini memecahkan rekor gol Prancis di Piala Dunia, Mbapp tampaknya belum selesai menulis sejarah. Dunia kini menanti satu pertanyaan besar: mampukah Kylian Mbapp mencetak tiga gol lagi dan merebut takhta Miroslav Klose sebagai pencetak gol terbanyak sepanjang sejarah Piala Dunia? Baca Juga : Mia Khalifa Bilang Foto Viralnya Nonton Piala Dunia Hasil AI Video: Ada Messi di Skuad Argentina untuk Piala Dunia 2026 Video: Ada Messi di Skuad Argentina untuk Piala Dunia 2026 (afr/afr) Tautan telah disalin TAGS piala dunia 2026 lionel messi miroslav klose timnas prancis trending topic gerd m ller mbappe kylian mbappe LIHAT LAINNYA</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Gibran: Indonesia Harus Jadi Penguasa AI, Bukan Sekedar Pengguna</t>
+          <t>Ponsel Tak Lagi Jadi Raja? CEO Qualcomm Ungkap Penggantinya</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Gibran: Indonesia Harus Jadi Penguasa AI, Bukan Sekedar Pengguna</t>
+          <t>Ponsel Tak Lagi Jadi Raja? CEO Qualcomm Ungkap Penggantinya</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/law-and-policy/d-8534648/gibran-indonesia-harus-jadi-penguasa-ai-bukan-sekedar-pengguna</t>
+          <t>https://inet.detik.com/business/d-8534792/ponsel-tak-lagi-jadi-raja-ceo-qualcomm-ungkap-penggantinya</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/law-and-policy/d-8534648/gibran-indonesia-harus-jadi-penguasa-ai-bukan-sekedar-pengguna</t>
+          <t>https://inet.detik.com/business/d-8534792/ponsel-tak-lagi-jadi-raja-ceo-qualcomm-ungkap-penggantinya</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/16/wakil-presiden-gibran-rakabuming-raka-1781619885697_43.png?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2025/10/29/ilustrasi-kirim-chat-atau-pesan-via-whatsapp-wa-1761720050538_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F11" s="1" t="n">
-        <v>46190.45775707352</v>
+        <v>46190.52412886219</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Jakarta - Qualcomm sedang mengembangkan lebih dari 40 desain perangkat AI baru, ungkap CEO Cristiano Amon, seiring persiapan perusahaan perancang chip tersebut dalam menyambut gelombang agen"AI di seluruh perangkat elektronik konsumen. "Saya rasa akan ada banyak eksperimen dengan berbagai bentuk perangkat (form factor). Saat ini, kami memiliki lebih dari 40 desain perangkat tersebut, dan saya katakan kepada Anda, variasi bentuknya sangat, sangat beragam," kata Amon yang dikutip detikINET dari CNBC. SCROLL TO CONTINUE WITH CONTENT Baca juga: Google Ubah Android Jadi 'Agen' AI yang Bisa Bertindak Sendiri Amon menyebut perangkat teknologi yang dapat dikenakan (wearable) ini mencakup perhiasan, earbuds yang dilengkapi kamera, pin, dan jam tangan. ADVERTISEMENT "Prinsipnya adalah sesuatu yang Anda kenakan, sesuatu yang selalu bersama Anda setiap saat, sesuatu yang dapat melihat dunia di sekitar Anda, sehingga Anda memiliki konteks dan kemampuan untuk mengakses serta berkomunikasi dengan agen," ujarnya. Agen (AI) dipandang sebagai evolusi selanjutnya asisten digital seperti Siri milik Apple atau Gemini dari Google. Industri teknologi bertaruh agen-agen ini akan mampu menjalankan tugas lebih panjang dan kompleks melintasi berbagai aplikasi dan layanan, seperti memesan tiket liburan. Amon memberikan contoh tentang agen yang mengambil detail transaksi perbankan, sehingga pengguna tidak perlu menavigasi aplikasi dan mencari secara manual. Ini menandakan cara kita berinteraksi dengan aplikasi akan berubah drastis di masa depan, ketika agen mengambil alih pelaksanaan tugas. "Aplikasi tidak mati tetapi aplikasi akan berubah. Agen-agen itulah yang akan menjadi aplikasi baru," tambahnya. CEO Qualcomm Cristiano Amon Foto: undefined Menjamurnya agen AI dan berubahnya cara kita menggunakan aplikasi di masa depan juga dapat mengubah interaksi orang dengan smartphone, serta menciptakan peluang bagi jenis perangkat baru untuk meledak. Agen AI bersiap mengganti HP sebagai pusat kehidupan digital. "Ponsel akan berpusat di sekitar agen. Kelas perangkat yang baru juga akan berpusat pada agen. Dan agen inilah yang akan memahami niat manusia dan akan melakukan banyak hal untuk Anda, jadi ada pergeseran mengenai apa yang menjadi titik pusatnya," jelas Amon, seraya menambahkan ponsel takkan menghilang sepenuhnya. Ia optimis terhadap kacamata pintar yang berpotensi menyaingi smartphone. Pengiriman kacamata pintar saat ini puluhan juta"per tahun. Beberapa tahun ke depan Amon memprediksi angkanya ratusan juta dan sebesar pasar HP. Sebagai perbandingan, terdapat 1,26 miliar smartphone dikirimkan pada 2025 menurut riset Counterpoint, naik sekitar 3% dibanding tahun sebelumnya. Berbagai perusahaan raksasa, mulai Meta hingga Samsung, saat ini berlomba mengembangkan kacamata pintar. Pergeseran lanskap perangkat dapat membuka pintu bagi jenis perusahaan baru untuk bersaing di pasar hardware konsumen. Tahun lalu, OpenAI mengakuisisi io, startup yang didirikan desainer Apple, Jony Ive, untuk merambah pasar perangkat konsumen. Motivasi lain di balik masuknya pemain baru di sektor hardware adalah penguasaan data. Amon mengatakan perangkat-perangkat ini akan mengumpulkan data jauh lebih besar dibandingkan data yang digunakan untuk melatih model AI. "Jadi perusahaan-perusahaan tersebut menginginkan akses ke data itu, karena hal tersebut penting untuk melatih model di masa depan sekaligus menciptakan pengalaman AI yang dibuat khusus bagi penggunanya," ungkap Amon. Baca juga: Terungkap! Ini Wujud Kacamata Pintar Samsung Pesaing Meta Ray-Ban RedMagic 11 Pro, Performa Ekstrim Ponsel Gaming! RedMagic 11 Pro, Performa Ekstrim Ponsel Gaming! (fyk/afr) TAGS pengganti smartphone qualcomm kacamata pintar agen ai interaksi digital perangkat wearable ponsel smartphone LIHAT LAINNYA Tautan telah disalin</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update project dependencies and generate missing node_modules files
</commit_message>
<xml_diff>
--- a/Pertemuan4/hasil_cleaning.xlsx
+++ b/Pertemuan4/hasil_cleaning.xlsx
@@ -460,350 +460,350 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>10 Foto Lionel Messi Hattrick, Dipuji Setinggi Langit</t>
+          <t>Heboh! Aplikasi Peta Ini Ungkap Data Rahasia Wilayah Korea Utara</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>10 Foto Lionel Messi Hattrick, Dipuji Setinggi Langit</t>
+          <t>Heboh! Aplikasi Peta Ini Ungkap Data Rahasia Wilayah Korea Utara</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/fotoinet/d-8535031/lionel-messi-hattrick-dipuji-setinggi-langit</t>
+          <t>https://inet.detik.com/cyberlife/d-8543091/heboh-aplikasi-peta-ini-ungkap-data-rahasia-wilayah-korea-utara</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/fotoinet/d-8535031/lionel-messi-hattrick-dipuji-setinggi-langit</t>
+          <t>https://inet.detik.com/cyberlife/d-8543091/heboh-aplikasi-peta-ini-ungkap-data-rahasia-wilayah-korea-utara</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/17/meme-messi-1781666958944_43.png?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2025/09/03/kereta-yang-dinaiki-kim-jong-un-dari-korea-utara-menuju-beijing-chnia-untuk-menghadiri-parade-militer-1756891002533_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F2" s="1" t="n">
-        <v>46190.52412886219</v>
+        <v>46196.52444533166</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Jakarta - Lionel Messi mencetak hattrick dalam kemenangan Argentina atas Aljazair 3-0 di ajang Piala Dunia 2026. Dengan 3 gol yang disarangkan ke Aljazair, Lionel Messi menjadi pencetak gol terbanyak di Piala Dunia bersama Miroslav Klose. Foto: X.com Messi dan Klose di puncak dengan sama-sama melesakkan 17 gol sepanjang sejarah keikutsertaan mereka di Piala Dunia. Foto: X.com Memang benar-benar Lionel Messi adalah pesepakbola terbaik dunia sampai saat ini. Foto: X.com Sungguh penampilan klasik dari Messi. Foto: X.com Sudah berusia 38 tahun dan memenangkan segalanya, Messi tadi tetap ngotot bahkan membantu pertahanan. Foto: X.com Akun resmi Timnas Argentina memuji penampilan sang mega bintang. Foto: X.com Messi pun menjadi Man of The Match. Foto: X.com Berbagai rekor menakjubkan Messi di ajang Piala Dunia. Foto: X.com Sudah 20 tahun berlalu, Messi tetap luar biasa. Foto: X.com Para megabintang mulai bersinar di Piala Dunia 2026. Foto: X.com (/) TAGS lionel messi piala dunia 2026 LIHAT LAINNYA Tautan telah disalin</t>
+          <t>Jakarta - Aplikasi peta digital, Kakao Map, bikin heboh di dunia maya setelah pengguna internet menemukan layanan tersebut menampilkan informasi geografis Korea Utara paling rahasia ke publik. Tentunya, informasi tersebut menjadi viral di berbagai platform media sosial karena banyak pengguna membandingkan data yang tersedia di Kakao Map dengan layanan pemetaan internasional yang selama ini memiliki keterbatasan dalam menampilkan informasi wilayah Korea Utara. Berdasarkan laporan The Korea Times, pengguna internet membagikan tangkapan layar yang menunjukkan berbagai informasi geografis di Korea Utara, mulai dari nama lokasi, fasilitas publik, hingga detail kawasan yang jarang terlihat di aplikasi peta global. SCROLL TO CONTINUE WITH CONTENT ADVERTISEMENT Baca Juga : Krisis Populasi Makin Parah, Korea Selatan Bentuk Tentara AI Popularitas unggahan tersebut memicu rasa penasaran publik karena Korea Utara dikenal sebagai salah satu negara paling tertutup di dunia dengan akses informasi yang sangat terbatas. Maka tak heran, selama ini data geografis yang rinci mengenai negara yang dipimpin Kim Jong Un itu jarang tersedia secara luas untuk masyarakat internasional. Kakao Map sendiri merupakan salah satu layanan pemetaan terbesar di Korea Selatan yang mengandalkan data lokal untuk menyediakan navigasi dan informasi lokasi secara detail. Platform ini selama bertahun-tahun menjadi alternatif utama bagi warga Korea Selatan selain layanan peta domestik lainnya. Viralnya data Korea Utara di Kakao Map juga muncul di tengah perhatian terhadap isu pemetaan digital di Korea Selatan. Sebelumnya, pemerintah Korea Selatan dikenal menerapkan berbagai pembatasan terhadap distribusi data peta berpresisi tinggi karena pertimbangan keamanan nasional dan sensitivitas hubungan dengan Korea Utara. Baca Juga : Antartika Geger, Peneliti Korea Ancam Rekan dengan Pisau Video: Timnas Korut U-17 Viral Beri 'Salam Pukul' ke Jepang di Piala Dunia Video: Timnas Korut U-17 Viral Beri 'Salam Pukul' ke Jepang di Piala Dunia (agt/afr) TAGS kakao map peta digital korea utara data rahasia media sosial LIHAT LAINNYA Tautan telah disalin</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Kampus Ini Sudah Lahirkan 12 Unicorn AI dan Hardware, Ada DJI di Baliknya</t>
+          <t>Messi Jadi Top Skor Piala Dunia Sepanjang Masa, Google Ikut Berpesta</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Kampus Ini Sudah Lahirkan 12 Unicorn AI dan Hardware, Ada DJI di Baliknya</t>
+          <t>Messi Jadi Top Skor Piala Dunia Sepanjang Masa, Google Ikut Berpesta</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8534903/kampus-ini-sudah-lahirkan-12-unicorn-ai-dan-hardware-ada-dji-di-baliknya</t>
+          <t>https://inet.detik.com/cyberlife/d-8543090/messi-jadi-top-skor-piala-dunia-sepanjang-masa-google-ikut-berpesta</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8534903/kampus-ini-sudah-lahirkan-12-unicorn-ai-dan-hardware-ada-dji-di-baliknya</t>
+          <t>https://inet.detik.com/cyberlife/d-8543090/messi-jadi-top-skor-piala-dunia-sepanjang-masa-google-ikut-berpesta</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/15/innox-1781527712161_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/21/undav-meledak-dan-samai-messi-perebutan-top-skor-pildun-2026-makin-panas-1782004747819_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F3" s="1" t="n">
-        <v>46190.52412886219</v>
+        <v>46196.52444533166</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Jakarta - Jika Silicon Valley dikenal sebagai rumah bagi raksasa teknologi dunia, China memiliki Shenzhen sebagai pusat lahirnya inovasi hardware dan kecerdasan buatan (AI). Di kota inilah berdiri Shenzhen InnoX Academy, sebuah institusi yang dijuluki banyak kalangan sebagai "pabrik startup" karena berhasil melahirkan puluhan perusahaan teknologi dengan dampak global. Didirikan pada 2021 oleh Profesor Li Zexiang, akademisi dari Hong Kong University of Science and Technology (HKUST) yang juga dikenal sebagai salah satu tokoh di balik kesuksesan DJI, InnoX mengusung konsep berbeda dari kampus atau inkubator startup konvensional. Mereka menggabungkan pendidikan kewirausahaan, inkubasi startup, akselerasi manufaktur, hingga dukungan ekspansi global dalam satu ekosistem terintegrasi. "Rekam jejak Li Zexiang sendiri tidak main-main. Selama kariernya, ia telah membantu menginkubasi lebih dari 200 perusahaan smart hardware yang menghasilkan empat perusahaan publik dan 12 unicorn, termasuk DJI yang kini menjadi pemimpin pasar drone konsumen dunia," terang Carol Yu Founding Partner &amp; Senior Vice President InnoX. SCROLL TO CONTINUE WITH CONTENT ADVERTISEMENT Baca Juga : Baseus PicoGo Air Rilis, Powerbank Setipis Kartu Tantang Xiaomi UltraThin Sejak berdiri, InnoX telah menarik lebih dari 19.000 pendaftar dari berbagai negara dan mendukung hampir 1.000 entrepreneur melalui berbagai program inovasi dan inkubasi startup. Saat ini, sekitar 100 proyek startup sedang dibina, dengan lebih dari 80% berfokus pada pengembangan AI dan hardware untuk pasar global. Model yang diterapkan InnoX berfokus pada membantu inovator mengubah ide menjadi produk siap pasar. Para peserta tidak hanya belajar teori bisnis, tetapi juga menjalani proses lengkap mulai dari riset pengguna, perancangan produk, pengembangan teknologi, pembuatan prototipe, hingga strategi pemasaran global. Sosok Profesor Li Zexiang Foto: Innox Keunggulan terbesar InnoX terletak pada lokasinya yang berada di Shenzhen, kota yang dikenal sebagai pusat manufaktur teknologi dunia. Melalui jaringan lebih dari 1.600 pemasok dan mitra manufaktur, startup dapat mempercepat proses pengembangan produk, menguji berbagai prototipe, hingga melakukan produksi massal dengan lebih cepat dibanding banyak negara lain. Tak hanya membantu membangun produk, InnoX juga mendorong startup untuk langsung berpikir global sejak hari pertama. Lebih dari 80% startup binaannya memang dirancang untuk pasar internasional. Dukungan yang diberikan mencakup strategi crowdfunding, pameran teknologi internasional, branding, akses investor, hingga jaringan bisnis global. Carol Yu Founding Partner &amp; Senior Vice President InnoX. Foto: Innox Kekuatan ekosistem tersebut terlihat dari beragam startup yang lahir dari InnoX. Mulai dari Kamingo yang mampu mengubah sepeda biasa menjadi e-bike dalam hitungan detik, XBREW dengan mesin kopi nitro tanpa kartrid pertama di dunia, hingga Y-H2O yang mengembangkan kapal hydrofoil listrik futuristis. Ada pula Finnox yang mengembangkan AI untuk memahami emosi manusia, serta Lumi, robot lampu berbasis AI yang menghadirkan interaksi layaknya karakter animasi Pixar. Pada ajang BEYOND Expo 2026, InnoX membawa sekitar 30 startup AI dan hardware untuk memamerkan inovasi terbaru mereka di bidang robotika, mobilitas pintar, embodied AI, kesehatan digital, hingga perangkat gaya hidup cerdas. Untuk memperkuat ekosistem inovasinya, InnoX juga menjalin kolaborasi dengan lebih dari 20 universitas ternama dunia, termasuk Stanford University, Olin College of Engineering, King Abdullah University of Science and Technology (KAUST), University of Hong Kong, dan HKUST. Jaringan global tersebut membuka akses bagi para pendiri startup ke talenta, investor, industri, serta sumber daya manufaktur dari berbagai negara. Innox Foto: Innox Di tengah persaingan global membangun dominasi AI, Shenzhen InnoX Academy menunjukkan bahwa kesuksesan tidak hanya ditentukan oleh teknologi canggih, tetapi juga oleh ekosistem yang mampu mengubah ide menjadi produk yang benar-benar digunakan masyarakat. "Dari Shenzhen, berbagai startup AI dan hardware kini bersiap menembus pasar dunia," pungkas Yu. Baca Juga : Tamagotchi Kini Makin Pintar, Punya AI dan Bisa Pantau Tanaman Video AI Bikin Konsumsi Air Dunia Melejit: Dampaknya Bisa Kekeringan! Video AI Bikin Konsumsi Air Dunia Melejit: Dampaknya Bisa Kekeringan! (afr/afr) TAGS unicorn shenzhen innox academy dji innox academy kecerdasan buatan startup teknologi global connect show LIHAT LAINNYA Tautan telah disalin</t>
+          <t>Jakarta - Lionel Messi kembali menorehkan tinta emas dalam sejarah sepak bola dunia. Kapten Timnas Argentina itu kini resmi menjadi pencetak gol terbanyak sepanjang masa di ajang Piala Dunia setelah melampaui rekor legenda Jerman, Miroslav Klose. Pencapaian bersejarah tersebut terjadi saat Argentina mengalahkan Austria dengan skor 2-0 dalam laga Grup J Piala Dunia 2026. Dua gol yang dicetak Messi membuat koleksi golnya di Piala Dunia bertambah menjadi 18 gol, melewati torehan 16 gol milik Klose yang bertahan selama lebih dari satu dekade. SCROLL TO CONTINUE WITH CONTENT Baca Juga : Mbappe Lewati Messi, 15 Gol Piala Dunia Tercepat Tuai Pujian Selangit ADVERTISEMENT Gol pertama Messi pada pertandingan tersebut menjadi momen pemecahan rekor. Tak berhenti di situ, La Pulga kembali mencetak gol pada masa injury time untuk semakin memperlebar jarak di puncak daftar top skor sepanjang masa Piala Dunia. Kehebatan Messi tak hanya mendapat sorotan dari penggemar sepak bola. Google juga ikut merayakan pencapaian luar biasa tersebut lewat fitur spesial yang muncul di mesin pencari mereka. Ketika pengguna mengetikkan kata kunci "Lionel Messi", "Messi" atau La Pulga di Google Search, layar langsung dihiasi efek visual meriah. Konfeti berwarna kuning dan biru yang identik dengan Argentina berjatuhan dari bagian atas halaman pencarian. Tak lama kemudian muncul animasi bola sepak dengan tulisan "All-time World Cup goal record holder!" yang menegaskan status baru Messi sebagai pemegang rekor gol terbanyak sepanjang sejarah Piala Dunia. Google rayakan Leonel Messi jadi top skor Piala Dunia sepanjang masa. Foto: Screenshoot Google juga menyediakan tombol konfeti interaktif yang bisa diklik pengguna. Setiap klik akan memunculkan hujan konfeti baru sekaligus menambah jumlah reaksi dari para penggemar. Hingga saat ini, jumlah reaksinya telah mencapai 6 jutaan dan terus bertambah. Fitur interaktif ini mirip dengan perayaan Google saat momen-momen ikonik lainnya, seperti kemenangan Argentina di Piala Dunia 2022. Kali ini, Google memberikan penghormatan langsung kepada Messi yang terus menunjukkan performa luar biasa meski sudah mendekati usia 39 tahun. Seperti diketahui, Messi sudah menyamai rekor Klose saat mencetak hat-trick ke gawang Aljazair pada laga pembuka Argentina di Piala Dunia 2026. Namun pertandingan melawan Austria menjadi momen yang benar-benar mengukuhkan dirinya sendirian di puncak daftar pencetak gol terbanyak turnamen empat tahunan tersebut. Rekor ini semakin melengkapi sederet pencapaian luar biasa Messi sepanjang kariernya. Setelah menjuarai Piala Dunia 2022, meraih berbagai gelar bersama klub dan tim nasional, kini pemain berusia 38 tahun itu kembali mencatat sejarah yang mungkin akan sulit dipecahkan dalam waktu dekat. Dengan Argentina yang tampil meyakinkan di fase grup dan berstatus juara bertahan, peluang Messi untuk menambah koleksi golnya masih terbuka lebar. Baca Juga : Messi Ukir 4 Rekor Baru Piala Dunia Sekaligus, Status GOAT Kian Kokoh Saksikan Live DetikPagi: Video: Ada Messi di Skuad Argentina untuk Piala Dunia 2026 Video: Ada Messi di Skuad Argentina untuk Piala Dunia 2026 (afr/afr) TAGS lionel messi top skor piala dunia rekor gol piala dunia 2026 la pulga google LIHAT LAINNYA Tautan telah disalin</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Zuckerberg Bayar Rp 248 T untuk Bocah Ajaib, Hasilnya Belum Ada</t>
+          <t>Tecno Camon Slim Meluncur, HP 6,39 mm dengan LED Kreatif Unik</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Zuckerberg Bayar Rp 248 T untuk Bocah Ajaib, Hasilnya Belum Ada</t>
+          <t>Tecno Camon Slim Meluncur, HP 6,39 mm dengan LED Kreatif Unik</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/business/d-8534912/zuckerberg-bayar-rp-248-t-untuk-bocah-ajaib-hasilnya-belum-ada</t>
+          <t>https://inet.detik.com/consumer/d-8543081/tecno-camon-slim-meluncur-hp-6-39-mm-dengan-led-kreatif-unik</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/business/d-8534912/zuckerberg-bayar-rp-248-t-untuk-bocah-ajaib-hasilnya-belum-ada</t>
+          <t>https://inet.detik.com/consumer/d-8543081/tecno-camon-slim-meluncur-hp-6-39-mm-dengan-led-kreatif-unik</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2025/06/11/alexandr-wang-1749622991230_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/23/tecno-camon-slim-1782177580666_43.png?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F4" s="1" t="n">
-        <v>46190.52412886219</v>
+        <v>46196.52444533166</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Jakarta - Sekitar setahun lampau, MarkZuckerberg berinvestasi gila-gilaan untuk meningkatkan kemampuan kecerdasan buatan atau AI Meta, yang tertinggal jauh dari pesaing. Salah satunya dengan merekrut pakar AIAlexandr Wang yang menghabiskan USD 14 miliar (Rp 248 triliun). Uang itu diguyur untuk Scale AI, startup AI yang didirikan oleh Wang, anak muda yang baru berusia 29 tahun saat ini tapi dianggap sangat cerdas di bidang AI. Beberapa engineer Scale AI juga bergabung dengan Meta. Pencapaian besar Wang yang memimpin MetaSuperintelligence Labs adalah peluncuran model AI Muse Spark bulan April. Dengan produk itu, Meta setidaknya kembali diperhitungkan di ranah AI, meskipun masih tertinggal jauh di belakang OpenAI, Anthropic, dan Google. Namun demikian dari sisi finansial, hasilnya belum ada. SCROLL TO CONTINUE WITH CONTENT Kini CEO Mark Zuckerberg bertugas menjadikan kerja keras Wang sebagai kesuksesan finansial. Itu berarti menunjukkan perusahaan mampu menarik pengguna berbayar untuk AI-nya. Baca juga: Curhat Karyawan Meta yang Dipindah ke Divisi AI: Seperti Gulag "Meta perlu memberi lebih banyak bukti nyata terkait adopsi maupun komersialisasi. Investor menantikan Meta memonetisasi produk baru yang mengutamakan AI, di luar dampak positif substansial yang diberikan AI dalam menyempurnakan model periklanan," ujar Ralph Schackart, analis di William Blair yang dikutip detikINET dari CNBC. ADVERTISEMENT Wall Street juga sejauh ini tidak terkesan. Saham Meta anjlok 18% 12 bulan terakhir. Hal itu terjadi bahkan setelah Meta melaporkan pertumbuhan pendapatan 33% pada kuartal pertama. Meta awalnya terjun ke ranah AI dengan model Llama, menawarkan pendekatan open source yang memungkinkan pengembang mengutak-atik secara bebas, sementara pembuat AI lain memungut biaya. Ternyata model itu adalah blunder. April 2025, peluncuran Llama 4 gagal total, tak mampu memikat pengembang dan membuat Zuckerberg mempertimbangkan kembali pendekatan AI Meta. Dua bulan kemudian, Zuckerberg mengejutkan dunia teknologi dengan mengumumkan investasi USD 14,3 miliar untuk Scale AI dan mendatangkan Wang. Pengembangan dan peluncuran Muse Spark oleh Wang pada bulan April tahun ini mulai menggerakkan roda perusahaan. Model baru ini dirancang mudah diintegrasikan ke aplikasi Meta seperti Facebook dan Instagram, serta perangkat AI seperti kacamata Ray-Ban Meta. Sebaik apapun model Wang, jalan Zuckerberg terjal setelah kegagalan Llama. "Saya rasa komunitas AI sebagian besar mengabaikan Meta pada titik ini," ujar Rob May, CEO startup Neurometric. Andrew Moore, CEO startup korporat Lovelace dan mantan kepala AI Google Cloud, mengatakan belum terlambat bagi Meta untuk menemukan jalurnya. Meta harus menunjukkan keunggulan di suatu area AI, entah itu pada biaya atau nuansa teknis lainnya yang penting bagi para pengembang. Masalah lain adalah kemerosotan moral kerja. Meta baru saja memecat sekitar 8.000 pekerja. Terdapat pula ketegangan di petinggi organisasi AI tersebut. Meskipun perilisan Muse Spark dinilai tinggi secara internal, ada tekanan yang dialami Wang bersama mantan CEO GitHub Nat Friedman, yang juga bergabung dengan Meta. Namun dalam podcast bulan Mei, Wang menepis konflik internal. Wang menyebut Muse Spark sebagai 'makanan pembuka"'untuk apa yang akan datang, dan mengatakan bahwa akan ada model-model yang lebih kuat. Baca juga: Pentolan AI Amerika Ramai Pindah ke China, Ada Apa? Video Top 5: TAEMIN Masuk Grammy Museum-Zuckerberg Jadi Penasihat Trump Video Top 5: TAEMIN Masuk Grammy Museum-Zuckerberg Jadi Penasihat Trump (fyk/fyk) TAGS mark zuckerberg alexandr wang LIHAT LAINNYA Tautan telah disalin</t>
+          <t>Jakarta - Tecno resmi memperkenalkan Camon Slim, smartphone terbaru yang mengandalkan desain ultra tipis dan fitur pencahayaan unik sebagai daya tarik utama. Dengan ketebalan hanya 6,39 mm, perangkat ini menjadi salah satu ponsel paling ramping yang pernah dirilis Tecno. Camon Slim hadir dengan desain curved unibody yang memberikan kesan premium sekaligus nyaman digenggam. Tecno juga menawarkan sejumlah pilihan warna dan finishing yang berbeda untuk menonjolkan karakter masing-masing pengguna. Varian New Mondrian menjadi yang paling mencuri perhatian. Bagian belakangnya mengusung pola khas Mondrian dan dilapisi material photochromic yang dapat berubah tampilan saat terkena sinar ultraviolet. Efek tersebut memunculkan blok warna kuning, hijau, dan cyan yang membuat ponsel terlihat lebih hidup. SCROLL TO CONTINUE WITH CONTENT ADVERTISEMENT Baca Juga : Tecno Pova 8 5G Bawa Baterai 8.000 mAh dan Layar 144Hz, Rilis di RI? Selain itu, tersedia pilihan Prism Black dan Jungle Green yang menggunakan pola 3D crystal diamond. Sementara varian Van Gogh Blue menghadirkan reproduksi lukisan legendaris Starry Night dengan sentuhan tekstur matte yang elegan. Varian Tecno Camon Slim Foto: Tecno Tak hanya mengandalkan penampilan, Tecno Camon Slim juga dibekali sertifikasi IP68 dan IP69. Dengan sertifikasi tersebut, perangkat ini memiliki ketahanan tinggi terhadap debu serta cipratan air bertekanan tinggi. Salah satu fitur paling menarik dari Camon Slim adalah panel LED yang terintegrasi di area kamera belakang. Tecno menyematkan 354 LED yang dapat menampilkan berbagai efek pencahayaan kreatif. LED tersebut telah dikonfigurasi dengan 55 skenario pencahayaan berbeda. Pengguna dapat memanfaatkannya untuk menambah efek visual saat mengambil foto dan video, menciptakan suasana tertentu ketika membuat konten, hingga berfungsi sebagai lampu notifikasi yang lebih atraktif dibandingkan LED konvensional. Tecno Camon Slim Foto: Tecno Untuk urusan performa, Tecno membekali Camon Slim dengan chipset MediaTek Helio G200 yang dipadukan RAM 8 GB. Kapasitas penyimpanan tersedia dalam pilihan 128 GB dan 256 GB. Di bagian depan terdapat layar berukuran 6,78 inci dengan resolusi 1224 x 2720 piksel serta refresh rate 144Hz. Kombinasi ini menjanjikan tampilan yang tajam dan animasi yang lebih mulus saat bermain game maupun scrolling media sosial. Sektor fotografi mengandalkan kamera utama 50 MP yang menggunakan sensor Sony Lytia 600 berukuran 1/2 inci. Untuk kebutuhan swafoto dan video call, tersedia kamera depan 32 MP. Tecno Camon Slim Foto: Tecno Meski memiliki bodi sangat tipis, Tecno tetap menyematkan baterai berkapasitas 5.600 mAh yang didukung pengisian cepat 60W. Tecno menyebut Camon Slim akan dipasarkan secara bertahap di berbagai negara. Namun hingga saat ini perusahaan belum mengungkap harga resmi maupun jadwal peluncurannya di Indonesia. Baca Juga : Tecno Spark 50 Resmi Masuk Indonesia, HP Rp 1 Jutaan Baterai 7.000 mAh Video Top 5: Konser BTS Jakarta Jadi 3 Hari hingga BGN Evaluasi MBG Video Top 5: Konser BTS Jakarta Jadi 3 Hari hingga BGN Evaluasi MBG (afr/afr) TAGS tecno camon slim smartphone tipis mediatek helio g200 LIHAT LAINNYA Tautan telah disalin</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>WhatsApp di iPhone Kini Bisa Pakai 2 Nomor Sekaligus, Begini Caranya</t>
+          <t>10 Foto Tim IT Menangis! Foto-foto Instalasi Kabel Ini Bikin Geleng Kepala</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>WhatsApp di iPhone Kini Bisa Pakai 2 Nomor Sekaligus, Begini Caranya</t>
+          <t>10 Foto Tim IT Menangis! Foto-foto Instalasi Kabel Ini Bikin Geleng Kepala</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/consumer/d-8534891/whatsapp-di-iphone-kini-bisa-pakai-2-nomor-sekaligus-begini-caranya</t>
+          <t>https://inet.detik.com/fotoinet/d-8543055/tim-it-menangis-foto-foto-instalasi-kabel-ini-bikin-geleng-kepala</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/consumer/d-8534891/whatsapp-di-iphone-kini-bisa-pakai-2-nomor-sekaligus-begini-caranya</t>
+          <t>https://inet.detik.com/fotoinet/d-8543055/tim-it-menangis-foto-foto-instalasi-kabel-ini-bikin-geleng-kepala</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2025/05/30/ilustrasi-menggunakan-smartphone-atau-whataapp-1748579035406_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/23/instalasi-kabel-bikin-tim-it-menangis-1782176504867_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F5" s="1" t="n">
-        <v>46190.52412886219</v>
+        <v>46196.52444533166</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Daftar Isi Cara Menambahkan Akun WhatsApp Kedua di iPhone Cara Beralih Antar Akun Keunggulan Fitur Multi-Akun WhatsApp Jakarta - abar gembira bagi pengguna iPhone. WhatsApp kini resmi menghadirkan fitur multi-akun di iOS yang memungkinkan pengguna menggunakan dua nomor telepon berbeda dalam satu aplikasi WhatsApp. Sebelumnya, pengguna iPhone yang ingin memakai dua akun WhatsApp biasanya harus mengandalkan WhatsApp Business atau aplikasi pihak ketiga. Kini, WhatsApp menghadirkan solusi resmi yang lebih praktis, aman, dan mudah digunakan. Fitur ini sangat berguna bagi pengguna yang ingin memisahkan akun pribadi dan pekerjaan tanpa harus berganti perangkat atau memasang aplikasi tambahan. Seluruh chat, notifikasi, hingga pengaturan privasi masing-masing akun akan tetap terpisah. SCROLL TO CONTINUE WITH CONTENT ADVERTISEMENT Baca Juga : WhatsApp Cabut Dukungan untuk iOS Lawas Ini, Segera Update iPhone Kalian! Dengan hadirnya fitur multi-akun, pengguna cukup berpindah akun langsung dari aplikasi WhatsApp tanpa perlu login dan logout berulang kali. Sebelum mencoba fitur ini, ada beberapa syarat yang perlu dipenuhi. Pengguna harus menggunakan WhatsApp versi terbaru yang sudah mendukung multi-akun di iOS. Selain itu, diperlukan dua nomor telepon aktif yang bisa berasal dari kombinasi SIM fisik dan eSIM, atau dua eSIM sekaligus. Cara Menambahkan Akun WhatsApp Kedua di iPhone Bagi yang ingin mencoba, berikut langkah-langkah menambahkan akun WhatsApp kedua di iPhone: Buka aplikasi WhatsApp di iPhone. Masuk ke menu Pengaturan (Settings). Ketuk bagian profil yang menampilkan nama dan nomor telepon. Pilih opsi Tambahkan Akun (Add Account). Masukkan nomor telepon kedua yang ingin digunakan. Lakukan proses verifikasi melalui SMS atau panggilan suara. Masukkan kode verifikasi yang diterima. Setelah proses selesai, akun kedua akan langsung aktif di aplikasi WhatsApp. Pengguna kini dapat menggunakan dua akun WhatsApp berbeda dalam satu aplikasi tanpa perlu menginstal aplikasi tambahan. Cara Beralih Antar Akun WhatsApp juga membuat proses perpindahan akun menjadi sangat mudah. Untuk berpindah akun: Buka menu Settings. Pada bagian atas akan muncul daftar akun yang aktif. Pilih akun yang ingin digunakan. Selain itu, pengguna juga bisa menekan lama tab Settings untuk berpindah akun dengan lebih cepat. Setiap akun memiliki pengaturan sendiri, termasuk notifikasi, status, foto profil, pengaturan privasi, hingga cadangan chat. Dengan begitu, aktivitas pribadi dan pekerjaan tetap dapat dipisahkan dengan rapi. Keunggulan Fitur Multi-Akun WhatsApp Kehadiran fitur ini membawa sejumlah keuntungan bagi pengguna iPhone, di antaranya: Tidak perlu lagi menggunakan aplikasi pihak ketiga yang berisiko terhadap keamanan data. Notifikasi untuk masing-masing akun tetap terpisah. Pengaturan privasi dapat diatur berbeda untuk setiap akun. Status, foto profil, dan tema bisa dikelola secara independen. Didukung langsung oleh WhatsApp sehingga lebih aman dan stabil. Meski demikian, ada beberapa hal yang perlu diperhatikan. Setiap akun tetap membutuhkan nomor telepon yang berbeda karena satu nomor hanya dapat digunakan untuk satu akun WhatsApp. Selain itu, fitur multi-akun diluncurkan secara bertahap. Jika opsi Tambahkan Akun belum muncul di perangkat, pengguna disarankan memperbarui aplikasi WhatsApp melalui App Store dan menunggu distribusi fitur tersedia untuk seluruh pengguna. Dengan hadirnya fitur multi-akun resmi di iPhone, pengguna kini dapat mengelola dua nomor WhatsApp dalam satu aplikasi secara lebih praktis. Fitur ini menjadi solusi yang selama ini ditunggu banyak pengguna iPhone yang ingin memisahkan urusan pribadi dan pekerjaan tanpa ribet. Baca Juga : WhatsApp Garap Fitur Scam Alert untuk Hindarkan Pengguna dari Penipuan Video: Instagram, Facebook, sampai WhatsApp Nggak Full Gratis Lagi? Video: Instagram, Facebook, sampai WhatsApp Nggak Full Gratis Lagi? (afr/afr) TAGS whatsapp iphone aplikasi whatsapp fitur baru whatsapp multi akun whatsapp LIHAT LAINNYA Tautan telah disalin</t>
+          <t>Jakarta - Deretan foto instalasi kabel paling semrawut yang pernah ditemukan. Bikin geleng kepala, bahkan tim IT dan teknisi berpengalaman pun bisa stres melihatnya. Ruang server ini lebih mirip semangkuk mi kusut raksasa. Mencari satu kabel yang bermasalah di sini mungkin butuh keberanian dan doa. Foto: Boredpanda Kabel listrik menembus sudut tembok tanpa pelindung memadai. Solusi cepat yang bisa membuat teknisi keselamatan sulit tidur. Foto: Boredpanda Ketika satu-satunya dokumentasi sistem adalah secarik kertas bertuliskan Jangan cabut apa pun . Tim IT langsung berkeringat dingin. Foto: Boredpanda Siapa sangka rak server dan toilet bisa berbagi ruangan? Kombinasi yang membuat konsep manajemen risiko kehilangan makna. Foto: Boredpanda Puluhan laptop diisi daya sekaligus dengan kabel berserakan di lantai. Satu langkah ceroboh saja bisa mengubah ruangan jadi arena domino elektronik. Foto: Boredpanda Teknisi ini tampak seperti sedang bertarung melawan monster kabel yang tumbuh liar di tiang utilitas kota. Foto: Boredpanda Panel listrik ini terlihat seperti teka-teki yang dibuat untuk menguji kesabaran manusia. Salah sentuh sedikit, konsekuensinya bisa mahal. Foto: Boredpanda Kotak distribusi jaringan ini seolah menyerah pada keteraturan. Kabel menjuntai ke segala arah tanpa ada yang benar-benar tahu ujungnya di mana. Foto: Boredpanda Sambungan kabel jaringan ini terlihat seperti proyek seni modern. Sayangnya, karya seni bukanlah fungsi utama sebuah jaringan. Foto: Boredpanda Saat pintu kabinet dibuka, yang terlihat bukan perangkat telekomunikasi melainkan mimpi buruk kolektif para teknisi lapangan. Foto: Boredpanda (/) TAGS fotoinet fotodetikcom LIHAT LAINNYA Tautan telah disalin</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tak Sabar Tunggu GTA 6, Pria Ini Bikin Tiruannya Pakai AI</t>
+          <t>Mbappe Lewati Messi, 15 Gol Piala Dunia Tercepat Tuai Pujian Selangit</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tak Sabar Tunggu GTA 6, Pria Ini Bikin Tiruannya Pakai AI</t>
+          <t>Mbappe Lewati Messi, 15 Gol Piala Dunia Tercepat Tuai Pujian Selangit</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/games-news/d-8534872/tak-sabar-tunggu-gta-6-pria-ini-bikin-tiruannya-pakai-ai</t>
+          <t>https://inet.detik.com/cyberlife/d-8543043/mbappe-lewati-messi-15-gol-piala-dunia-tercepat-tuai-pujian-selangit</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/games-news/d-8534872/tak-sabar-tunggu-gta-6-pria-ini-bikin-tiruannya-pakai-ai</t>
+          <t>https://inet.detik.com/cyberlife/d-8543043/mbappe-lewati-messi-15-gol-piala-dunia-tercepat-tuai-pujian-selangit</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2025/05/07/rockstar-rilis-trailer-gta-6-yang-kedua-tampilkan-aksi-2-karakter-utama-1746583798227_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/17/kylian-mbappe-1781648830427_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F6" s="1" t="n">
-        <v>46190.52412886219</v>
+        <v>46196.52444533166</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Jakarta - Grand Theft Auto (GTA) 6 dijadwalkan meluncur pada November 2026 setelah dikembangkan kurang lebih satu dekade. Namun, seorang pendiri startup sudah tidak sabar menunggu lebih lama dan memutuskan membuat game tiruan GTA 6 dengan bantuan AI. Ziwen Xu, pendiri startup Hyperecho, belum lama ini mengumumkan rencananya untuk membuat GTA 6 versinya sendiri dengan teknik vibe coding. Ia menggunakan Claude 20x, model AI generatif paling canggih dari Anthropic yang tersedia untuk publik. Proyek itu dimulainya pada 11 Juni kemarin. Sejak saat itu, Xu terus membagikan update terbaru tentang kemajuan proyeknya dan membagikan kodenya di GitHub jika ada orang lain yang ingin melanjutkan proyeknya. SCROLL TO CONTINUE WITH CONTENT Baca Juga : Demi Info Terbaru Game GTA 6, YouTuber Mau Bobol Kantor Rockstar "Targetnya: mengalahkan peluncuran GTA 6 yang sebenarnya. Ambisius, mungkin bodoh, tapi saya tetap akan melakukannya," tulis Xu dalam postingannya di X, seperti dikutip dari Gizmodo, Rabu (17/6/2026). ADVERTISEMENT [Gambas:Twitter] Postingan yang diunggah Xu di X menyertakan cuplikan video singkat dari game tersebut. Pada hari pertama, sebagian besar cuplikan gameplay-nya hanya terdiri dari oval biru 3D yang bergerak dan melompat-lompat di dekat balok abu-abu. Di hari kedua, Xu mengunggah video baru yang menunjukkan karakter yang bentuknya mulai mirip seperti manusia sedang berlarian di lanskap perkotaan. Namun, Xu mengakui bahwa itu masih jauh dari sempurna. "Agen AI membangun gedung pencakar langit di pusat kota LA, yang jadi masalah besar, karena (game) ini seharusnya di Florida," tulis Xu. "Selain itu, saya telah menghabiskan 33% dari penggunaan mingguan 20x saya dalam satu hari. Jadi waktu terus berjalan," sambungnya. Hari keenam setelah proyek ini dimulai, game buatan Xu sudah terlihat lebih ekspansif dengan karakter NPC yang berjalan-jalan, mobil di jalanan, dan bahkan senjata. GTA 6 baru akan diluncurkan pada bulan November, jadi Xu masih memiliki beberapa bulan untuk menyelesaikan proyek game-nya dan mengalahkan developer Rockstar Games. Belum diketahui sejauh mana komitmen Xu untuk melanjutkan proyek game ini. Baca Juga : GTA 6 Dominasi November 2026, Banyak Game Besar Pilih Menjauh Video Pesan Wapres Gibran untuk Generasi Muda: Gunakan AI untuk Belajar Video Pesan Wapres Gibran untuk Generasi Muda: Gunakan AI untuk Belajar (vmp/afr) TAGS gta 6 ai vibe coding LIHAT LAINNYA Tautan telah disalin</t>
+          <t>Jakarta - Kylian Mbappe kembali menyumbang satu gol saat laga Prancis vs Irak di Piala Dunia 2026. Ini merupakan gol ke-15 Mbappe di Piala Dunia, dan ia mampu mengalahkan Lionel Messi dalam hal kecepatan mencapai angka tersebut. Messi memang saat ini berada di posisi puncak sebagai pemain dengan jumlah gol terbanyak di Piala Dunia dengan 18 gol, namun Mbappe berhasil menjadi yang tercepat dalam meraih 15 gol di ajang tersebut. Penyerang andalan Prancis itu hanya membutuhkan 16 pertandingan untuk mencetak 15 gol di Piala Dunia. Sebagai perbandingan, Messi memerlukan 27 pertandingan untuk mencapai jumlah gol yang sama. Catatan tersebut semakin menegaskan ketajaman Mbappe di panggung sepak bola terbesar dunia. SCROLL TO CONTINUE WITH CONTENT ADVERTISEMENT Baca Juga : Messi Ukir 4 Rekor Baru Piala Dunia Sekaligus, Status GOAT Kian Kokoh Badai Petir Gol bersejarah itu lahir saat Prancis menghadapi Irak pada laga kedua Grup I yang berlangsung di Philadelphia Stadium, Selasa (23/6/2026) dini hari WIB. Dilansir dari detikSport, sejak menit awal, Les Bleus tampil dominan dan menguasai jalannya pertandingan. Prancis akhirnya membuka keunggulan pada menit ke-14 melalui aksi Mbappe. Gol bermula dari kerja sama apik dengan Michael Olise di sisi kanan serangan. Mbappe kemudian menusuk ke area pertahanan Irak sebelum melepaskan tembakan kaki kiri yang meluncur deras ke pojok kanan atas gawang. Gol tersebut membuat Prancis unggul 1-0 sekaligus mengukir catatan baru dalam perjalanan karier Mbappe di Piala Dunia. Setelah unggul, Prancis terus mengendalikan permainan. Penguasaan bola mereka mencapai sekitar 60 persen sepanjang babak pertama. Irak dibuat kesulitan mengembangkan permainan dan jarang menciptakan peluang berbahaya. Peluang terbaik Irak datang melalui sundulan Ali Alhamadi yang memanfaatkan umpan Merchas Doski. Namun bola masih melebar dari sasaran. Beberapa kesempatan melalui tendangan sudut juga gagal dimaksimalkan untuk membobol gawang Prancis. Ketika pertandingan memasuki jeda babak pertama dengan keunggulan Prancis 1-0, situasi tak terduga terjadi. Badai petir yang melanda kawasan Philadelphia membuat kickoff babak kedua harus ditunda demi alasan keselamatan. Dari dalam stadion, layar besar menampilkan peringatan cuaca ekstrem dan meminta para penonton meninggalkan kursi tribune. "Badai petir hebat sedang mendekat," demikian bunyi pesan yang ditampilkan di Stadion Philadelphia. Pemerintah setempat juga mengeluarkan peringatan banjir akibat hujan lebat dan badai besar yang melanda wilayah tersebut. [Gambas:Twitter] Pujian Selangit Sementara pertandingan babak kedua masih ditunda, pencapaian Mbappe langsung menjadi perbincangan hangat di media sosial. Banyak penggemar sepak bola memuji kemampuan sang penyerang yang terus menunjukkan konsistensi luar biasa di Piala Dunia. Meski Messi masih memegang rekor gol terbanyak sepanjang sejarah Piala Dunia dengan 18 gol, laju Mbappe yang sudah mencapai 15 gol hanya dalam 16 pertandingan membuat banyak pihak yakin bahwa pemain Prancis itu berpeluang besar menambah koleksi golnya dan terus mendekati berbagai catatan legendaris milik La Pulga. "Dunia karena dia mungkin akan bermain di Piala Dunia berikutnya dan pasti akan mencetak beberapa gol lagi di Piala Dunia ini," kata @tsrakasu9. "Rekor yang luar biasa di Piala Dunia. Dia pasti akan menjadi pencetak gol terbanyak," ucap @AdamBoor11. "Kylian Mbapp adalah talenta murni tanpa gembar-gembor, berada di posisi ketiga bersama Ronaldo dalam daftar pencetak gol terbanyak Piala Dunia.," ujar @Sevenhappy007. "Anak muda ini sedang dalam performa terbaik. 15 gol Piala Dunia dan satu gol untuk Prancis. Pencetak gol terbanyak sepanjang masa Prancis dengan 59 gol dan terus bertambah. Dia diam-diam membangun warisannya sendiri meskipun usianya masih muda, dan masih banyak lagi yang akan datang," kata @okafor_nna54678. "Pemain Piala Dunia terhebat sepanjang masa. Kylian Mbappe. Tidak seperti pemain curang yang mencetak 18 gol dalam 6 pertandingan Piala Dunia, sebagian besar melalui penalti," sindir @Utd_Rico. Baca Juga : Mbappe Lampaui Messi di Piala Dunia, Netizen Doakan Pecahkan Rekor Klose Saksikan Live DetikPagi: Video: Ada Messi di Skuad Argentina untuk Piala Dunia 2026 Video: Ada Messi di Skuad Argentina untuk Piala Dunia 2026 (afr/afr) Tautan telah disalin TAGS kylian mbappe piala dunia 2026 gol tercepat lionel messi rekor gol sepak bola prancis LIHAT LAINNYA</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>15 Foto Hanya Mata Jeli yang Bisa Menemukan Sosok di Foto 'Penampakan' Ini</t>
+          <t>Ingat! Aturan Daftar Nomor HP Baru Berlaku Pekan Depan</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15 Foto Hanya Mata Jeli yang Bisa Menemukan Sosok di Foto 'Penampakan' Ini</t>
+          <t>Ingat! Aturan Daftar Nomor HP Baru Berlaku Pekan Depan</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/fotoinet/d-8534856/hanya-mata-jeli-yang-bisa-menemukan-sosok-di-foto-penampakan-ini</t>
+          <t>https://inet.detik.com/law-and-policy/d-8543024/ingat-aturan-daftar-nomor-hp-baru-berlaku-pekan-depan</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/fotoinet/d-8534856/hanya-mata-jeli-yang-bisa-menemukan-sosok-di-foto-penampakan-ini</t>
+          <t>https://inet.detik.com/law-and-policy/d-8543024/ingat-aturan-daftar-nomor-hp-baru-berlaku-pekan-depan</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/17/kumpulan-foto-unik-dengan-sosok-tersembunyi-yang-sulit-ditemukan-1781658346072_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2025/11/26/ilustrasi-face-recognition-1764163471563_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F7" s="1" t="n">
-        <v>46190.52412886219</v>
+        <v>46196.52444533166</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Jakarta - Kumpulan foto unik dengan sosok tersembunyi yang sulit ditemukan. Uji ketelitian mata dan lihat apakah kamu bisa menemukannya lebih cepat dari orang lain. Pemilik rumah ini mengaku akhirnya berhasil membeli rumah impiannya setelah bertahun-tahun menabung. Namun ada satu detail aneh di dapur mungil ini yang langsung menarik perhatian netizen. Apakah kamu menemukannya? Foto: Boredpanda Sekilas hanya terlihat kebun biasa yang dipenuhi rumput liar. Padahal ada seekor hewan yang bersembunyi dengan kamuflase nyaris sempurna di dalam foto ini. Foto: Boredpanda Foto ruang kuliah ini tampak normal, tetapi ada satu sosok yang membuat banyak orang harus melihatnya dua kali sebelum sadar apa yang sebenarnya terjadi. Foto: Boredpanda Batuan bersalju ini terlihat seperti tebing biasa. Namun jika diamati lebih teliti, ada penghuni liar yang menyatu hampir sempurna dengan lingkungan sekitarnya. Foto: Boredpanda Tas ransel hitam ini sukses membuat banyak orang bingung. Bukan karena bentuknya, melainkan karena ada sesuatu yang tersembunyi di dekatnya. Foto: Boredpanda Ekskavator CAT ini tampak seperti alat berat biasa yang sedang diparkir. Namun ada hewan berhasil bersembunyi di tempat yang tidak terduga. Foto: Boredpanda Rimbunnya daun bambu membuat objek tersembunyi dan berbahaya dalam foto ini sangat sulit ditemukan. Hanya mata yang benar-benar jeli yang bisa melihatnya dalam hitungan detik. Foto: Boredpanda Tumpukan kaus kaki ini ternyata menyimpan kejutan. Ada sepasang mata yang mengintip dari balik lipatan kain dan membuat foto ini viral. Foto: Boredpanda Pemandangan desa yang indah dari udara ini menyimpan satu objek yang tidak seharusnya ada di sana. Banyak orang baru menyadarinya setelah diperbesar. Foto: Boredpanda Hutan kering ini tampak kosong tanpa penghuni. Faktanya, ada seekor hewan yang sedang mengawasi kamera sambil berkamuflase dengan sangat baik. Foto: Boredpanda Kucing hitam ini sebenarnya tidak sendirian. Banyak orang baru menyadarinya setelah melihat bagian matanya yang menyala. Foto: Boredpanda Pagar kayu dan tanaman rambat tampak biasa saja. Tapi ada seekor ular yang berkamuflase begitu sempurna hingga sulit ditemukan dalam sekali pandang. Foto: Boredpanda Daun hijau ini menyimpan penghuni tersembunyi yang nyaris tak terlihat. Bentuk dan warnanya begitu mirip dengan daun tempat ia hinggap. Foto: Boredpanda Seorang pedagang roti sedang melayani pelanggan di pinggir jalan. Namun ada 'penjaga toko' tak terduga yang bersembunyi di etalase dan membuat banyak orang tertipu. Foto: Boredpanda Hamparan bebatuan dan dedaunan kering ini ternyata bukan sekadar pemandangan hutan biasa. Seekor ular besar bersembunyi di depan kamera dengan kamuflase yang luar biasa. Foto: Boredpanda (/) TAGS fotoinet fotodetikcom LIHAT LAINNYA Tautan telah disalin</t>
+          <t>Jakarta - Aturan pendaftaran registrasi SIM card prabayar baru menggunakan data pengenalan wajah atau face recognition akan berlaku pekan depan, yakni tepatnya 1 Juli 2026. Kebijakan teranyar Komdigi ini akan menggantikan sistem pendaftaran nomor HP baru sebelumnya yang menggunakan data nomor induk kependudukan (NIK) dan nomor kartu keluarga (KK) yang masih belum menangkal penyalahgunaan nomor seluler hingga penipuan online. Sosialisasi aturan tersebut telah dilakukan selama enam bulan terhitung sejak awal tahun. Komdigi memastikan registrasi SIM card baru yang divalidasi data biometrik akan diterapkan pada 1 Juli 2026. SCROLL TO CONTINUE WITH CONTENT Baca Juga : Ancaman Hak Kekayaan Intelektual Makin Masif, Komdigi Perkuat Pengawasan ADVERTISEMENT Direktur Jenderal Ekosistem Digital Kementerian Komdigi, Edwin Hidayat Abdullah mengatakan kepastian itu berdasarkan uji coba yang dilakukan pemerintah bersama operator seluler, Indosat Ooredoo Hutchison, Telkomsel, dan XLSmart. Disampaikannya, ketiga operator seluler tersebut dinyatakan mumpuni untuk melayani pendaftaran nomor HP baru pakai pengenalan wajah. "Jadi, per 1 Juli 2026 akan diterapkan secara nasional," ujar Edwin dalam konferensi pers di Garuda Sparks, Jakarta beberapa waktu lalu. Kewajiban penggunaan data biometrik menggunakan wajah pengguna ini tertuang dalam Peraturan Menteri Komunikasi dan Digital Nomor 7 Tahun 2026 tentang Registrasi Pelanggan Jasa Telekomunikasi melalui Jaringan Bergerak Seluler. Kewajiban perekaman wajah tersebut ditujukan untuk yang akan mengaktifkan nomor seluler prabayar terbaru, sedangkan pelanggan eksisting bersifat sukarela. Sedangkan, pelanggan yang di bawah 17 tahun atau belum memiliki identitas pribadi, maka dapat diwakilkan melalui data orang tua atau wali. Seperti aturan sebelumnya, pemerintah menetapkan pembatasan maksimal tiga nomor seluler untuk setiap operator bagi satu identitas pelanggan, sehingga total masyarakat hanya memiliki sembilan nomor telepon seluler. Kebijakan ini bertujuan menekan praktik penyalahgunaan SIM card dalam jumlah besar. Adapun, registrasi SIM card pakai data perekaman wajah ini bisa dilakukan dengan dua cara, yaitu datang langsung ke gerai operator seluler yang prosesnya akan dipandu petugas atau registrasi mandiri (self-registration) melalui aplikasi atau situs web resmi operator. Komdigi menyebutkan bahwa data biometrik pelanggan tidak disimpan di database operator seluler. Operator hanya melakukan proses validasi (passthrough), sementara penyimpanan data berada di Direktorat Jenderal Dukcapil. Baca Juga : Warga Perbatasan Marak Pakai Starlink, Bakti: Bukan Pesaing Saksikan Live DetikPagi: Video: Arnold Ph. Djiwatampu Raih Best Lifetime Achiever Dunia Telekomunikasi Video: Arnold Ph. Djiwatampu Raih Best Lifetime Achiever Dunia Telekomunikasi (agt/afr) TAGS registrasi sim card pengenalan wajah data biometrik registrasi sim card biometrik registrasi sim card face recognition komdigi operator seluler LIHAT LAINNYA Tautan telah disalin</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Haaland Menggila di Debut Piala Dunia 2026, Borong 2 Gol Bikin Heboh Medsos</t>
+          <t>Messi Ukir 4 Rekor Baru Piala Dunia Sekaligus, Status GOAT Kian Kokoh</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Haaland Menggila di Debut Piala Dunia 2026, Borong 2 Gol Bikin Heboh Medsos</t>
+          <t>Messi Ukir 4 Rekor Baru Piala Dunia Sekaligus, Status GOAT Kian Kokoh</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8534834/haaland-menggila-di-debut-piala-dunia-2026-borong-2-gol-bikin-heboh-medsos</t>
+          <t>https://inet.detik.com/cyberlife/d-8543019/messi-ukir-4-rekor-baru-piala-dunia-sekaligus-status-goat-kian-kokoh</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8534834/haaland-menggila-di-debut-piala-dunia-2026-borong-2-gol-bikin-heboh-medsos</t>
+          <t>https://inet.detik.com/cyberlife/d-8543019/messi-ukir-4-rekor-baru-piala-dunia-sekaligus-status-goat-kian-kokoh</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/17/irak-vs-norwegia-1781650428426_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/23/lionel-messi-timnas-argentina-piala-dunia-2026-argentina-vs-austria-top-skor-piala-dunia-1782157290513_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F8" s="1" t="n">
-        <v>46190.52412886219</v>
+        <v>46196.52444533166</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Jakarta - Erling Haaland akhirnya mencatatkan debut yang sangat dinanti di Piala Dunia 2026. Striker andalan Norwegia itu langsung tampil menggila dengan mencetak dua gol saat membantu timnya meraih kemenangan meyakinkan 4-1 atas Irak pada laga Grup I. Penampilan Haaland langsung menjadi sorotan dunia sepak bola. Bomber Manchester City tersebut menunjukkan mengapa dirinya dianggap sebagai salah satu penyerang paling berbahaya di generasi saat ini. Dua gol yang dicetaknya membuat pertahanan lawan tak berkutik dan membawa Norwegia membuka langkah di Piala Dunia dengan hasil sempurna. Tak pelak media sosial ikut heboh membahas aksi sang striker yang untuk pertama kalinya tampil di ajang sepak bola paling bergengsi di dunia. SCROLL TO CONTINUE WITH CONTENT ADVERTISEMENT Baca Juga : Mbappe Lampaui Messi di Piala Dunia, Netizen Doakan Pecahkan Rekor Klose Tak butuh waktu lama, nama Haaland langsung merajai trending topic di berbagai platform media sosial. Warganet dari berbagai negara ramai membahas aksi sang striker yang langsung mencetak brace pada penampilan pertamanya di Piala Dunia. [Gambas:Twitter] Di X, ribuan komentar memuji ketajaman pemain berusia 25 tahun tersebut. "Mungkin Haaland bisa aja jadi top score nih," kata @Muhammad_MARG. "Monster memang. Kalo butuh striker yang ahli finishing, tipe kaya haland ini yang paling bagus. Fisik oke, finishing juga oke. Jadi kombinasi yang bisa nyusahin lawan. Striker yang pas flop pun minimal cetak 25+ gol semusim," ujar @primas110. "Keren banget emang terminator satu ini," puji @kawulabolaid. "Debut Piala Dunia? Dua gol dan tiga poin. Haaland tak membuang waktu untuk memperkenalkan dirinya kepada dunia. Panggung Piala Dunia adalah satu-satunya yang kurang dalam catatan prestasinya. Ia sudah mulai menebus waktu yang hilang," tulis @abi_mat1 Video cuplikan dua gol Haaland juga viral di TikTok dan Instagram. Berbagai editan video dengan musik dramatis serta julukan "The Cyborg" membanjiri lini masa dan mengumpulkan jutaan tayangan hanya dalam hitungan jam. Kemenangan atas Irak menjadi modal berharga bagi Norwegia untuk melangkah ke fase berikutnya. Kehadiran Haaland membuat harapan publik Norwegia semakin tinggi setelah sekian lama tim nasional mereka jarang menjadi sorotan di panggung dunia. Jika mampu mempertahankan performa seperti ini, bukan tidak mungkin Haaland akan menjadi salah satu bintang terbesar turnamen sekaligus pesaing serius dalam perebutan gelar top skor. Baca Juga : Arab Saudi Tahan Uruguay, Netizen: Tutorial Kalahkan Arab Ada di Timnas Indonesia Video: Norwegia Lolos ke Piala Dunia 2026, Kalahkan Italia 4-1 Video: Norwegia Lolos ke Piala Dunia 2026, Kalahkan Italia 4-1 (afr/afr) TAGS haaland piala dunia 2026 gol haaland norwegia trending topic media sosial manchester city LIHAT LAINNYA Tautan telah disalin</t>
+          <t>Jakarta - Lionel Messi kembali membuktikan bahwa usianya hanyalah angka. Kapten Timnas Argentina itu mencetak sejarah baru di Piala Dunia 2026 dengan memecahkan empat rekor sekaligus, sekaligus memperkuat statusnya sebagai GOAT (Greatest of All Time) di mata banyak pencinta sepak bola dunia. Momen bersejarah itu terjadi saat Argentina mengalahkan Austria 2-0 pada laga Grup J. Messi menjadi pahlawan kemenangan Albiceleste lewat dua gol yang dicetaknya pada menit ke-39 dan masa injury time babak kedua. Meski sempat gagal mengeksekusi penalti di awal laga, La Pulga tetap mampu menorehkan malam yang tak terlupakan. Dua gol tersebut membuat Messi resmi menjadi pencetak gol terbanyak sepanjang sejarah Piala Dunia dengan koleksi 18 gol. Ia melewati rekor lama milik legenda Jerman, Miroslav Klose, yang mengoleksi 16 gol. Messi kini berdiri sendirian di puncak daftar top skor sepanjang masa turnamen paling bergengsi di dunia itu. SCROLL TO CONTINUE WITH CONTENT ADVERTISEMENT Baca Juga : Messi Hat-trick, Ronaldo Mandul! Debat GOAT Kembali Membara Tak hanya memecahkan rekor top skor, Messi juga mencatatkan tiga rekor lain yang membuat namanya semakin sulit disaingi. Berdasarkan catatan Guinness World Records, pemain berusia 38 tahun itu kini menjadi: Pemain dengan jumlah pertandingan terbanyak di Piala Dunia dengan 28 laga Pemain dengan kemenangan terbanyak di Piala Dunia sebanyak 18 kemenangan Pemain dengan total menit bermain terbanyak sepanjang sejarah turnamen, yakni 2.489 menit. [Gambas:Twitter] Catatan tersebut menjadi bukti konsistensi luar biasa Messi selama enam edisi Piala Dunia sejak debutnya pada 2006. Hingga kini, ia masih menjadi sosok sentral dalam permainan Argentina dan terus tampil menentukan di saat tim membutuhkan. Lebih istimewa lagi, rekor ini tercipta ketika Argentina memastikan tiket ke babak gugur Piala Dunia 2026. Dengan turnamen yang masih berlangsung, peluang Messi untuk menambah koleksi gol dan memperlebar jarak dari para pesaingnya masih terbuka lebar. Daftar top skor sepanjang masa Piala Dunia kini dipimpin Messi dengan 18 gol, diikuti Miroslav Klose (16 gol), Ronaldo Nazario (15 gol), serta Kylian Mbappe dan Gerd Muller yang sama-sama mengoleksi 14 gol. [Gambas:Twitter] Reaksi Warganet Pencapaian Messi langsung memicu gelombang pujian dari seluruh dunia. Nama sang megabintang merajai trending topic media sosial, sementara banyak penggemar menyebut mereka sedang menyaksikan sejarah secara langsung. "Apa yang telah dicapai Lionel Messi di usia 38 tahun sungguh legendaris. Menjadi legenda Piala Dunia ke-6 bukan hanya soal bakat, tetapi juga tentang kerja keras selama puluhan tahun, ketahanan, dan gairah yang tak tertandingi terhadap permainan ini. Perdebatan telah resmi berakhir. Hidup Raja!" ujar @Larykul2. "Dan Messi baru memainkan 2 pertandingan di turnamen ini. Masih banyak pertandingan dan gol yang harus dicetak. Bersiaplah untuk lebih banyak rekor yang akan dipecahkan olehnya. Kita sedang menyaksikan Messi di puncak performanya, sang legenda. GOAT dan setara dengan Pele dan Maradona di jajaran legenda sepak bola," kata @bmartawardaya. "Messi sedang dalam perjalanan untuk mencetak rekor lain melawan Yordania. Jika dia mencetak gol, dia akan menjadi pemain pertama yang mencetak gol dalam 7 pertandingan Piala Dunia berturut-turut. Rekor yang luar biasa. " ujar @NathanielOkwusa. "Di usia 38 tahun, di Piala Dunia KEENAM-nya, masih menulis ulang seluruh buku sejarah. Gol terbanyak di final (18), pertandingan terbanyak (28), kemenangan terbanyak (18), menit bermain terbanyak (2.489). Ini bukan sekadar umur panjang, ini adalah LEGENDA . Kita tidak sedang menonton seorang pemain, kita sedang menyaksikan babak terakhir dari kisah terhebat yang pernah diceritakan dalam sepak bola. Terima kasih, Leo. Sang GOAT tidak pernah meninggalkan gedung," ucap @bodex333. Dari Ballon d'Or, Copa America, hingga trofi Piala Dunia, Messi sudah mengoleksi hampir semua pencapaian yang bisa diraih seorang pesepak bola. Kini, dengan empat rekor baru yang berhasil dipecahkan sekaligus, warisan La Pulga dalam sejarah sepak bola semakin abadi dan membuat status GOAT-nya kian kokoh. Bagaimana menurut detikers? Baca Juga : Mbappe Lampaui Messi di Piala Dunia, Netizen Doakan Pecahkan Rekor Klose Saksikan Live DetikPagi: Video: Ada Messi di Skuad Argentina untuk Piala Dunia 2026 Video: Ada Messi di Skuad Argentina untuk Piala Dunia 2026 (afr/afr) Tautan telah disalin TAGS messi piala dunia 2026 goat rekor sepak bola argentina la pulga top skor pencapaian messi LIHAT LAINNYA</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Gibran Ingatkan Bahaya AI, Singgung Teknologi Tanpa Etika Itu Berbahaya</t>
+          <t>Bos WhatsApp Mengundurkan Diri, Digantikan Pendiri Startup Asal India</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Gibran Ingatkan Bahaya AI, Singgung Teknologi Tanpa Etika Itu Berbahaya</t>
+          <t>Bos WhatsApp Mengundurkan Diri, Digantikan Pendiri Startup Asal India</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/law-and-policy/d-8534804/gibran-ingatkan-bahaya-ai-singgung-teknologi-tanpa-etika-itu-berbahaya</t>
+          <t>https://inet.detik.com/business/d-8543012/bos-whatsapp-mengundurkan-diri-digantikan-pendiri-startup-asal-india</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/law-and-policy/d-8534804/gibran-ingatkan-bahaya-ai-singgung-teknologi-tanpa-etika-itu-berbahaya</t>
+          <t>https://inet.detik.com/business/d-8543012/bos-whatsapp-mengundurkan-diri-digantikan-pendiri-startup-asal-india</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/17/gibran-rakabuming-1781653746966_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2019/01/19/c9ca4724-afd8-4be9-a0a7-7641be6c3907_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F9" s="1" t="n">
-        <v>46190.52412886219</v>
+        <v>46196.52444533166</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Jakarta - Wakil Presiden Gibran Rakabuming Raka mengingatkan bahwa pesatnya perkembangan kecerdasan buatan atau Artificial Intelligence (AI) harus diiringi dengan penerapan etika yang kuat. Di tengah semakin luasnya pemanfaatan AI di berbagai bidang, Gibran menilai masyarakat perlu memahami bahwa teknologi bukan hanya soal kemampuan teknis, tetapi juga soal nilai dan integritas dalam penggunaannya. Meski menekankan Indonesia harus menguasai teknologi AI di masa mendatang, namun ia menyoroti ada hal utama yang dikedepankan terkait teknologi canggih ini, yakni terkait etika. SCROLL TO CONTINUE WITH CONTENT ADVERTISEMENT Baca Juga : Pesan Gibran ke Pelajar: Gunakan AI untuk Belajar, Bukan untuk Malas "Ada satu hal yang jauh lebih penting dari sekedar teknis penguasaan AI, yaitu etika. Teknologi tanpa etika itu berbahaya," kata Gibran seperti dikutip dari akun Instagram miliknya gibran_rakabuming, Rabu (17/6/2026). Ia menjelaskan AI memiliki potensi besar untuk membantu manusia menciptakan berbagai inovasi dan konten positif. Namun di sisi lain, teknologi yang sama juga dapat disalahgunakan untuk menyebarkan informasi palsu, melakukan plagiarisme, hingga melanggar privasi orang lain. "AI bisa digunakan untuk membuat konten positif, tapi juga bisa dipakai untuk menyebar hoax, melakukan plagiarisme, atau melanggar privasi orang lain," ucapnya. Gibran mengingatkan generasi muda agar tidak menggunakan AI untuk tindakan yang merugikan orang lain, melainkan kecanggihan teknologi harus dimanfaatkan untuk memberikan manfaat bagi masyarakat, bukan sebaliknya. "Saya ingin mengingatkan, pemanfaatan AI harus didasari oleh nilai-nilai integritas. Jangan gunakan AI untuk menipu. Jangan gunakan AI untuk menjatuhkan orang lain," tegasnya. Gibran Rakabuming, Wakil Presiden RI Foto: YouTube/@GibranTV Gibran menilai tantangan terbesar dalam era AI bukan hanya bagaimana masyarakat menguasai teknologi tersebut, tetapi juga bagaimana memastikan teknologi digunakan secara bertanggung jawab. "AI harus digunakan untuk kesejahteraan bersama, untuk mempermudah hidup, bukan untuk menciptakan kekacauan sosial. Kemajuan teknologi harus berjalan beriringan dengan kemajuan moralitas kita sebagai bangsa yang beradab," katanya. Dalam kesempatan tersebut, Gibran menyebut Indonesia memiliki talenta-talenta terbaik di bidang AI. Untuk itu, dikatanya, pemerintah menyiapkan ekosistemnya. Gibran juga menyinggung langkah pemerintah dalam menyiapkan tata kelola AI yang bertanggung jawab, yakni Indonesia telah menyelesaikan Readiness Assessment Methodology (RAM) AI yang disusun UNESCO sebagai instrumen untuk menilai kesiapan sekaligus tata kelola AI nasional. "Kuasai teknologinya. Pegang teguh etikanya. Mari kita jadikan AI sebagai jembatan menuju Indonesia yang lebih maju, lebih cerdas, dan lebih bermartabat," pungkasnya. Baca Juga : Gibran: Indonesia Harus Jadi Penguasa AI, Bukan Sekedar Pengguna Video Pesan Wapres Gibran untuk Generasi Muda: Gunakan AI untuk Belajar Video Pesan Wapres Gibran untuk Generasi Muda: Gunakan AI untuk Belajar (agt/afr) TAGS gibran rakabuming gibran rakabuming raka etika ai kecerdasan buatan ai etika teknologi LIHAT LAINNYA Tautan telah disalin</t>
+          <t>Jakarta - Head of WhatsApp Will Cathcart mengundurkan diri setelah memimpin aplikasi milik Meta tersebut selama hampir tujuh tahun. Cathcart akan digantikan oleh Kunal Shah, pendiri startup fintech Cred asal India. Dalam unggahannya di X, Cathcart mengatakan saat ini WhatsApp berada dalam posisi paling kuat, tetapi ini adalah momen yang tepat untuk mundur. "Saya sangat bangga dengan apa yang telah kita bangun," tulis Cathcart dalam postingannya, seperti dikutip detikINET, Selasa (23/6/2026). SCROLL TO CONTINUE WITH CONTENT ADVERTISEMENT Baca Juga : Viral Arti Warna Contact WhatsApp, Hijau Tak Save Nomor Kamu? "Kita telah mengembangkan platform pesan terenkripsi end-to-end hingga menjangkau lebih dari tiga miliar orang. Kita menghadirkannya ke chat grup, perangkat pendamping, platform baru - dan mempertahankan hak orang-orang di seluruh dunia untuk melakukan percakapan private," sambungnya. Will Cathcart Foto: TNM Cathcart akan tetap bertahan di Meta, tapi posisi barunya tidak disebutkan. CEO Meta Mark Zuckerberg dalam postingannya di Facebook hanya mengatakan Cathcart akan mengembangkan produk baru di Meta dari awal. Dalam unggahan yang sama, Zuckerberg memuji Shah yang sukses mengembangkan Cred menjadi salah satu perusahaan teknologi penting di India. Ia mengatakan SHah memiliki mentalitas pembangun dan perspektif global yang akan membantunya memimpin WhatsApp. "Saya berharap dapat bekerja sama dengan Kunal untuk terus menjadikan WhatsApp sebagai layanan terbaik untuk miliaran orang dan jutaan bisnis," kata Zuckerberg, seperti dikutip dari BBC. Shah mendirikan Cred pada tahun 2018. Cred adalah platform pembayaran kartu kredit yang memberikan bonus kepada pengguna yang membayar tagihannya tepat waktu. Kunal Shah Foto: Ndtv Sebagai bagian dari penunjukan Shah sebagai bos baru WhatsApp, Meta akan menginvestasikan USD 900 juta di Cred. Shah akan mundur sebagai CEO Cred tapi ia tetap akan menjadi pemegang saham. Cathcart ditunjuk sebagai bos WhatsApp pada tahun 2019. Selama memimpin aplikasi perpesanan terbesar di dunia, ia memperkenalkan sejumlah perubahan besar seperti backup chat terenkripsi, aplikasi WhatsApp untuk iPad, menghadirkan iklan, hingga menambahkan chatbot Meta AI. Baca Juga : Moral Karyawan Meta Ambruk, Bos Janjikan Lebih Banyak Camilan Video: Instagram, Facebook, sampai WhatsApp Nggak Full Gratis Lagi? Video: Instagram, Facebook, sampai WhatsApp Nggak Full Gratis Lagi? (vmp/afr) TAGS whatsapp bos whatsapp meta LIHAT LAINNYA Tautan telah disalin</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mbappe Lampaui Messi di Piala Dunia, Netizen Doakan Pecahkan Rekor Klose</t>
+          <t>Khusus Android, Hapus Aplikasi Ini kalau Mau M-Banking Aman</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Mbappe Lampaui Messi di Piala Dunia, Netizen Doakan Pecahkan Rekor Klose</t>
+          <t>Khusus Android, Hapus Aplikasi Ini kalau Mau M-Banking Aman</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8534801/mbappe-lampaui-messi-di-piala-dunia-netizen-doakan-pecahkan-rekor-klose</t>
+          <t>https://inet.detik.com/security/d-8542724/khusus-android-hapus-aplikasi-ini-kalau-mau-m-banking-aman</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/cyberlife/d-8534801/mbappe-lampaui-messi-di-piala-dunia-netizen-doakan-pecahkan-rekor-klose</t>
+          <t>https://inet.detik.com/security/d-8542724/khusus-android-hapus-aplikasi-ini-kalau-mau-m-banking-aman</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2026/06/17/kylian-mbappe-1781642953407_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2025/08/23/ilustrasi-hacker-1755942985725_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F10" s="1" t="n">
-        <v>46190.52412886219</v>
+        <v>46196.52444533166</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Jakarta - Kylian Mbappe kembali membuktikan dirinya sebagai salah satu pemain terbaik dunia saat ini. Penyerang Timnas Prancis itu mencetak dua gol dalam kemenangan 3-1 atas Senegal pada laga pembuka Grup I Piala Dunia 2026, Rabu (17/6/2026) dini hari WIB. Brace tersebut bukan sekadar membantu Les Bleus meraih tiga poin penting. Mbappe juga resmi mencatatkan namanya dalam sejarah sebagai pencetak gol terbanyak Timnas Prancis di ajang Piala Dunia. Dua gol ke gawang Senegal membuat koleksi gol Mbappe di Piala Dunia mencapai 14 gol. Catatan itu membuatnya melampaui sejumlah legenda sepak bola dunia, termasuk Lionel Messi, sekaligus menyamai torehan legenda Jerman, Gerd M ller. SCROLL TO CONTINUE WITH CONTENT Baca Juga : Arab Saudi Tahan Uruguay, Netizen: Tutorial Kalahkan Arab Ada di Timnas Indonesia ADVERTISEMENT Kini, pemain berusia 27 tahun itu hanya terpaut dua gol dari Ronaldo Naz rio yang mengoleksi 15 gol dan tiga gol dari pemegang rekor sepanjang masa Piala Dunia, Miroslav Klose, dengan 16 gol. Tak hanya itu, dua gol ke gawang Senegal juga mengantarkan Mbappe mengoleksi 58 gol untuk Timnas Prancis. Jumlah tersebut membuatnya melampaui rekor Olivier Giroud sebagai pencetak gol terbanyak sepanjang sejarah Les Bleus. Gol ke gawang Senegal juga membuat Mbappe memperpanjang rekor uniknya. Ia kini berhasil mencetak gol dalam tiga edisi Piala Dunia secara beruntun, yakni 2018, 2022, dan 2026. Dengan format baru Piala Dunia yang diikuti 48 negara, setiap tim berpeluang memainkan lebih banyak pertandingan dibanding edisi sebelumnya. Situasi ini menjadi keuntungan tersendiri bagi Mbapp dalam perburuan rekor gol sepanjang masa. [Gambas:Twitter] Medsos Dibanjiri Pujian Penampilan gemilang sang kapten langsung memicu reaksi besar di media sosial. Nama Mbapp menjadi salah satu topik yang ramai diperbincangkan usai laga hingga masuk daftar trending topic dunia. Banyak penggemar menyebutnya sebagai pemain yang sedang menuju status legenda sepak bola dunia. Banyak yang mendoakan Mbappe memecahkan rekor terbanyak di dunia sepanjang masa. "3 GOL lagi melampaui gol Misroslav Klose dan jadi pencetak gol terbanyak Pildun sepanjang masa!," ujar @naufaldzimam. "Messi sama ronaldo bener2 ga ada apa2nya dibanding mbappe kalo urusan performa di piala dunia. Messi paling top di 2014. Mbappe ni kayaknya bakal 3x turnamen 3x menggila," kata @nararay__. "Gile baru 27 tahun udah jadi topskor Prancis sepanjang masa, kalo melangkah jauh di pildun ini bisa lewatin gol nya klose juga nih," ucap @hendrasumar. "Gap Klose-Mbapp tinggal 2 gol aja , perancis punya mesin gol yg nggak main main ," kata @Suri_Ethan. Kylian Mbapp mencetak dua gol saat Prancis mengalahkan Senegal 3-1 Foto: Getty Images/Dan Mullan Jika Prancis mampu melaju hingga babak akhir turnamen, Mbapp berpotensi menambah koleksi golnya dan melampaui catatan Miroslav Klose yang selama ini dianggap sulit disentuh. Melihat usianya yang masih 27 tahun, peluang Mbapp bahkan tidak hanya terbuka di Piala Dunia 2026. Ia masih berpotensi tampil pada edisi berikutnya dan memperlebar rekor tersebut. Setelah menjadi juara dunia pada 2018, meraih Sepatu Emas pada 2022, dan kini memecahkan rekor gol Prancis di Piala Dunia, Mbapp tampaknya belum selesai menulis sejarah. Dunia kini menanti satu pertanyaan besar: mampukah Kylian Mbapp mencetak tiga gol lagi dan merebut takhta Miroslav Klose sebagai pencetak gol terbanyak sepanjang sejarah Piala Dunia? Baca Juga : Mia Khalifa Bilang Foto Viralnya Nonton Piala Dunia Hasil AI Video: Ada Messi di Skuad Argentina untuk Piala Dunia 2026 Video: Ada Messi di Skuad Argentina untuk Piala Dunia 2026 (afr/afr) Tautan telah disalin TAGS piala dunia 2026 lionel messi miroslav klose timnas prancis trending topic gerd m ller mbappe kylian mbappe LIHAT LAINNYA</t>
+          <t>Jakarta - Ada trik licik lagi dari hacker jahat untuk menjebak pengguna Android yang ingin download aplikasi terkenal. Mereka menggunakan bug yang dinamai Rokarolla yang bila sekali saja diinstal, bakal jadi malware yang sangat berbahaya. Rokarolla dapat memata-matai (spy) perangkat dan bahkan mencuri data pribadi yang sensitif, termasuk banking login. Bahkan, dia punya kemampuan membuat lockscreen palsu overlay untuk menangkap PIN, pattern keamanan, hingga password. Melansir Mirror , Selasa (23/6/2026), kasus terkait Rokarolla pertama kali dideteksi oleh tim dari Zimperium. Jadi, orang-orang yang kena jebakan ini bermula dari kemampuan Android untuk menginstal aplikasi dari sumber eksternal (sideloading) ke perangkat. Ini adalah fitur yang sangat disukai dari Android, yang merupakan sistem operasi yang lebih terbuka daripada iOS milik Apple. SCROLL TO CONTINUE WITH CONTENT Baca Juga : Hati-hati! Wallpaper Anime Dipakai Sebarkan Malware Pencuri Data ADVERTISEMENT Ketika orang mencari aplikasi, misalnya TikTok atau Chrome, mereka bakal diarahkan ke website palsu yang tampilannya kelihatan meyakinkan. Mirip tampilan resmi software. Jika tertipu, versi palsu aplikasi akan diunduh, bersamaan dengan penambahan Rokarolla di latar belakang. Aplikasi tersebut kemudian meminta sejumlah besar izin pribadi, seperti mengakses notifikasi. Karena semuanya tampak legal, mudah saja untuk terjebak mengklik 'iya'. Begitu itu terjadi, penjahat siber dapat mulai mencuri data. "Rokarolla menargetkan ekosistem yang luas yang terdiri dari lebih dari 200 aplikasi keuangan, mata uang kripto, dan media sosial," jelas Zimperium. "Dengan menggunakan taktik penghindaran yang canggih, ancaman ini secara khusus dirancang untuk menghindari solusi keamanan seluler berbasis tanda tangan yang sudah ada," imbuhnya. Cara terbaik untuk menghindari menjadi korban adalah hanya mengunduh aplikasi dari Google Play Store resmi. Penginstalan aplikasi dari sumber eksternal mungkin kadang dibutuhkan, tetapi mengunduh perangkat lunak dengan cara ini selalu disertai risiko. Ada baiknya juga untuk memastikan Google Play Protect diaktifkan. Google mengatakan perangkat akan terlindungi dari bug ini jika layanan ini diaktifkan. Baca Juga : 1 dari 5 Komputer Industri RI Diserang Malware, Sektor Migas Sasaran Empuk Saksikan Live DetikPagi: Video: Hati-hati! Ini Tandanya Jika Akun Gmail Sudah Diretas Video: Hati-hati! Ini Tandanya Jika Akun Gmail Sudah Diretas (ask/ask) TAGS malware rokarolla keamanan siber m-banking pencurian data google play store LIHAT LAINNYA Tautan telah disalin</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ponsel Tak Lagi Jadi Raja? CEO Qualcomm Ungkap Penggantinya</t>
+          <t>Berasa Gladiator, Elon Musk dan Zuckerberg Maunya Tarung di Koloseum</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Ponsel Tak Lagi Jadi Raja? CEO Qualcomm Ungkap Penggantinya</t>
+          <t>Berasa Gladiator, Elon Musk dan Zuckerberg Maunya Tarung di Koloseum</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/business/d-8534792/ponsel-tak-lagi-jadi-raja-ceo-qualcomm-ungkap-penggantinya</t>
+          <t>https://inet.detik.com/cyberlife/d-8542720/berasa-gladiator-elon-musk-dan-zuckerberg-maunya-tarung-di-koloseum</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/business/d-8534792/ponsel-tak-lagi-jadi-raja-ceo-qualcomm-ungkap-penggantinya</t>
+          <t>https://inet.detik.com/cyberlife/d-8542720/berasa-gladiator-elon-musk-dan-zuckerberg-maunya-tarung-di-koloseum</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2025/10/29/ilustrasi-kirim-chat-atau-pesan-via-whatsapp-wa-1761720050538_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2023/03/13/koloseum-bangunan-keajaiban-dan-ikon-kota-roma-italia-4_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F11" s="1" t="n">
-        <v>46190.52412886219</v>
+        <v>46196.52444533166</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Jakarta - Qualcomm sedang mengembangkan lebih dari 40 desain perangkat AI baru, ungkap CEO Cristiano Amon, seiring persiapan perusahaan perancang chip tersebut dalam menyambut gelombang agen"AI di seluruh perangkat elektronik konsumen. "Saya rasa akan ada banyak eksperimen dengan berbagai bentuk perangkat (form factor). Saat ini, kami memiliki lebih dari 40 desain perangkat tersebut, dan saya katakan kepada Anda, variasi bentuknya sangat, sangat beragam," kata Amon yang dikutip detikINET dari CNBC. SCROLL TO CONTINUE WITH CONTENT Baca juga: Google Ubah Android Jadi 'Agen' AI yang Bisa Bertindak Sendiri Amon menyebut perangkat teknologi yang dapat dikenakan (wearable) ini mencakup perhiasan, earbuds yang dilengkapi kamera, pin, dan jam tangan. ADVERTISEMENT "Prinsipnya adalah sesuatu yang Anda kenakan, sesuatu yang selalu bersama Anda setiap saat, sesuatu yang dapat melihat dunia di sekitar Anda, sehingga Anda memiliki konteks dan kemampuan untuk mengakses serta berkomunikasi dengan agen," ujarnya. Agen (AI) dipandang sebagai evolusi selanjutnya asisten digital seperti Siri milik Apple atau Gemini dari Google. Industri teknologi bertaruh agen-agen ini akan mampu menjalankan tugas lebih panjang dan kompleks melintasi berbagai aplikasi dan layanan, seperti memesan tiket liburan. Amon memberikan contoh tentang agen yang mengambil detail transaksi perbankan, sehingga pengguna tidak perlu menavigasi aplikasi dan mencari secara manual. Ini menandakan cara kita berinteraksi dengan aplikasi akan berubah drastis di masa depan, ketika agen mengambil alih pelaksanaan tugas. "Aplikasi tidak mati tetapi aplikasi akan berubah. Agen-agen itulah yang akan menjadi aplikasi baru," tambahnya. CEO Qualcomm Cristiano Amon Foto: undefined Menjamurnya agen AI dan berubahnya cara kita menggunakan aplikasi di masa depan juga dapat mengubah interaksi orang dengan smartphone, serta menciptakan peluang bagi jenis perangkat baru untuk meledak. Agen AI bersiap mengganti HP sebagai pusat kehidupan digital. "Ponsel akan berpusat di sekitar agen. Kelas perangkat yang baru juga akan berpusat pada agen. Dan agen inilah yang akan memahami niat manusia dan akan melakukan banyak hal untuk Anda, jadi ada pergeseran mengenai apa yang menjadi titik pusatnya," jelas Amon, seraya menambahkan ponsel takkan menghilang sepenuhnya. Ia optimis terhadap kacamata pintar yang berpotensi menyaingi smartphone. Pengiriman kacamata pintar saat ini puluhan juta"per tahun. Beberapa tahun ke depan Amon memprediksi angkanya ratusan juta dan sebesar pasar HP. Sebagai perbandingan, terdapat 1,26 miliar smartphone dikirimkan pada 2025 menurut riset Counterpoint, naik sekitar 3% dibanding tahun sebelumnya. Berbagai perusahaan raksasa, mulai Meta hingga Samsung, saat ini berlomba mengembangkan kacamata pintar. Pergeseran lanskap perangkat dapat membuka pintu bagi jenis perusahaan baru untuk bersaing di pasar hardware konsumen. Tahun lalu, OpenAI mengakuisisi io, startup yang didirikan desainer Apple, Jony Ive, untuk merambah pasar perangkat konsumen. Motivasi lain di balik masuknya pemain baru di sektor hardware adalah penguasaan data. Amon mengatakan perangkat-perangkat ini akan mengumpulkan data jauh lebih besar dibandingkan data yang digunakan untuk melatih model AI. "Jadi perusahaan-perusahaan tersebut menginginkan akses ke data itu, karena hal tersebut penting untuk melatih model di masa depan sekaligus menciptakan pengalaman AI yang dibuat khusus bagi penggunanya," ungkap Amon. Baca juga: Terungkap! Ini Wujud Kacamata Pintar Samsung Pesaing Meta Ray-Ban RedMagic 11 Pro, Performa Ekstrim Ponsel Gaming! RedMagic 11 Pro, Performa Ekstrim Ponsel Gaming! (fyk/afr) TAGS pengganti smartphone qualcomm kacamata pintar agen ai interaksi digital perangkat wearable ponsel smartphone LIHAT LAINNYA Tautan telah disalin</t>
+          <t>Jakarta - Sempat heboh tantangan duel MMA Elon Musk dan Mark Zuckerberg beberapa waktu silam. Kabar menyebut keduanya waktu itu sempat bersedia gelut, tapi di Koloseum, Italia. Kemungkinan, pertarungan di Koloseum tak bakal terwujud jika orangnya bukan mereka berdua, seperti dikatakan oleh CEO UFC Dana White. Dikutip detikINET dari TalkSport , Senin (22/6/2026), setelah pertunjukan spektakuler UFC di Gedung Putih akhir pekan lalu, Dana White ditanya apakah ia akan mempertimbangkan untuk menggelar pertarungan di tempat-tempat yang lebih ikonik. Misalnya Koloseum Roma. SCROLL TO CONTINUE WITH CONTENT Baca Juga : Mark Zuckerberg Nilai Elon Musk Tak Serius soal Duel ADVERTISEMENT White kemudian menjawab bahwa hal itu sulit dilakukan. Dulu, dia sempat negosiasi dengan Zuckerberg dan Musk soal hal itu, tapi tidak menjadi kenyataan. "Saya benar-benar berada di halaman belakang rumah saya selama dua minggu untuk menegosiasikan pertarungan itu, dan mereka menginginkan (pertarungan itu diadakan di) Koloseum," terang White. Kala itu, Koloseum menginginkan sekitar USD 150 juta untuk menyelenggarakannya di sana. Dana yang akan masuk bakal digunakan untuk memulihkan semua tempat ikonik di Italia. "Koloseum membutuhkan pertarungan antara Zuckerberg dan Musk agar pertarungan itu terjadi, karena keduanya akan menyediakan uang untuk mewujudkan pertarungan tersebut," ujarnya. Sebelumnya diceritakan bahwa Zuckerberg yang merupakan petarung yang sudah terlatih ini menunjukkan ketertarikannya naik kandang. Pada 2023, bos Meta itu setuju melawan Musk di 'pertandingan kandang'. Namun, setelah berbulan-bulan beredar rumor, pembicaraan tentang kemungkinan pertarungan itu meredup. Zuckerberg mengatakan Musk tidak serius tentang hal itu, dan menambahkan bahwa 'sudah waktunya untuk move on'. Selain klaim Zuckerberg bahwa Musk tidak mau berkomitmen, tampaknya tidak ada alasan lain mengapa pertarungan antara raksasa teknologi itu tidak pernah terwujud. Baca Juga : Elon Musk: Facebook Memanipulasi Publik Video Top 5: TAEMIN Masuk Grammy Museum-Zuckerberg Jadi Penasihat Trump Video Top 5: TAEMIN Masuk Grammy Museum-Zuckerberg Jadi Penasihat Trump (ask/ask) TAGS elon musk mark zuckerberg duel mma koloseum ufc LIHAT LAINNYA Tautan telah disalin</t>
         </is>
       </c>
     </row>

</xml_diff>